<commit_message>
Otomatik Veri Güncellemesi: Excel ve Yönetici Paneli Logları [Nispi Veri]
</commit_message>
<xml_diff>
--- a/Gorev-Listesi.xlsx
+++ b/Gorev-Listesi.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23676" windowHeight="10992" tabRatio="515"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23670" windowHeight="10995" tabRatio="515"/>
   </bookViews>
   <sheets>
     <sheet name="SES SERVİSİ ÇALIŞMA PLANI" sheetId="2" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="73">
   <si>
     <t>CUMA</t>
   </si>
@@ -224,9 +224,6 @@
     <t>A.C.PEHLİVAN.</t>
   </si>
   <si>
-    <t>PROVA</t>
-  </si>
-  <si>
     <t>CB Külliye   KURULUM</t>
   </si>
   <si>
@@ -237,6 +234,15 @@
   </si>
   <si>
     <t>???</t>
+  </si>
+  <si>
+    <t>HAZIRLIK</t>
+  </si>
+  <si>
+    <t>Çekmeköy Depo</t>
+  </si>
+  <si>
+    <t>KURULUM + PROVA</t>
   </si>
 </sst>
 </file>
@@ -1494,6 +1500,15 @@
     <xf numFmtId="49" fontId="11" fillId="4" borderId="9" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1527,15 +1542,6 @@
     <xf numFmtId="49" fontId="11" fillId="7" borderId="13" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="7" borderId="14" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1566,19 +1572,19 @@
     <xf numFmtId="49" fontId="11" fillId="9" borderId="13" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="14" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="15" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="9" borderId="16" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="9" borderId="8" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="9" borderId="9" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="9" borderId="14" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="9" borderId="15" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="9" borderId="16" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2031,7 +2037,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="175" row="2" locked="1">
+  <wetp:taskpane dockstate="right" visibility="1" width="350" row="1" locked="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -2057,56 +2063,56 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AR133"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="1.6640625" style="26" customWidth="1"/>
-    <col min="2" max="2" width="2.6640625" style="26" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" style="26" customWidth="1"/>
-    <col min="4" max="4" width="6.6640625" style="26" customWidth="1"/>
-    <col min="5" max="5" width="1.6640625" style="26" customWidth="1"/>
-    <col min="6" max="6" width="2.6640625" style="26" customWidth="1"/>
-    <col min="7" max="7" width="20.6640625" style="26" customWidth="1"/>
-    <col min="8" max="8" width="6.6640625" style="26" customWidth="1"/>
-    <col min="9" max="9" width="1.6640625" style="26" customWidth="1"/>
-    <col min="10" max="10" width="2.6640625" style="26" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="26" customWidth="1"/>
-    <col min="12" max="12" width="6.6640625" style="26" customWidth="1"/>
-    <col min="13" max="13" width="1.6640625" style="26" customWidth="1"/>
-    <col min="14" max="14" width="2.6640625" customWidth="1"/>
-    <col min="15" max="15" width="20.6640625" customWidth="1"/>
-    <col min="16" max="16" width="6.6640625" customWidth="1"/>
-    <col min="17" max="17" width="1.6640625" customWidth="1"/>
-    <col min="18" max="18" width="2.6640625" customWidth="1"/>
-    <col min="19" max="19" width="20.6640625" customWidth="1"/>
-    <col min="20" max="20" width="6.6640625" customWidth="1"/>
-    <col min="21" max="21" width="1.6640625" customWidth="1"/>
-    <col min="22" max="22" width="2.6640625" customWidth="1"/>
-    <col min="23" max="23" width="20.6640625" customWidth="1"/>
-    <col min="24" max="24" width="6.6640625" customWidth="1"/>
-    <col min="25" max="25" width="1.6640625" customWidth="1"/>
-    <col min="26" max="26" width="2.6640625" customWidth="1"/>
-    <col min="27" max="27" width="20.6640625" customWidth="1"/>
-    <col min="28" max="28" width="6.6640625" customWidth="1"/>
-    <col min="29" max="29" width="1.6640625" customWidth="1"/>
-    <col min="30" max="30" width="2.6640625" customWidth="1"/>
-    <col min="31" max="31" width="20.6640625" customWidth="1"/>
-    <col min="32" max="32" width="6.6640625" customWidth="1"/>
-    <col min="33" max="33" width="1.6640625" customWidth="1"/>
-    <col min="34" max="34" width="2.6640625" customWidth="1"/>
-    <col min="35" max="35" width="20.6640625" customWidth="1"/>
-    <col min="36" max="36" width="6.6640625" customWidth="1"/>
-    <col min="37" max="37" width="1.6640625" customWidth="1"/>
-    <col min="38" max="38" width="2.6640625" customWidth="1"/>
-    <col min="39" max="39" width="20.6640625" customWidth="1"/>
-    <col min="40" max="40" width="6.6640625" customWidth="1"/>
-    <col min="41" max="41" width="2.6640625" customWidth="1"/>
-    <col min="42" max="42" width="16.6640625" customWidth="1"/>
-    <col min="43" max="43" width="3.6640625" customWidth="1"/>
-    <col min="44" max="44" width="8.33203125" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" style="26" customWidth="1"/>
+    <col min="2" max="2" width="2.7109375" style="26" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="26" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" style="26" customWidth="1"/>
+    <col min="5" max="5" width="1.7109375" style="26" customWidth="1"/>
+    <col min="6" max="6" width="2.7109375" style="26" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="26" customWidth="1"/>
+    <col min="8" max="8" width="6.7109375" style="26" customWidth="1"/>
+    <col min="9" max="9" width="1.7109375" style="26" customWidth="1"/>
+    <col min="10" max="10" width="2.7109375" style="26" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" style="26" customWidth="1"/>
+    <col min="12" max="12" width="6.7109375" style="26" customWidth="1"/>
+    <col min="13" max="13" width="1.7109375" style="26" customWidth="1"/>
+    <col min="14" max="14" width="2.7109375" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" customWidth="1"/>
+    <col min="16" max="16" width="6.7109375" customWidth="1"/>
+    <col min="17" max="17" width="1.7109375" customWidth="1"/>
+    <col min="18" max="18" width="2.7109375" customWidth="1"/>
+    <col min="19" max="19" width="20.7109375" customWidth="1"/>
+    <col min="20" max="20" width="6.7109375" customWidth="1"/>
+    <col min="21" max="21" width="1.7109375" customWidth="1"/>
+    <col min="22" max="22" width="2.7109375" customWidth="1"/>
+    <col min="23" max="23" width="20.7109375" customWidth="1"/>
+    <col min="24" max="24" width="6.7109375" customWidth="1"/>
+    <col min="25" max="25" width="1.7109375" customWidth="1"/>
+    <col min="26" max="26" width="2.7109375" customWidth="1"/>
+    <col min="27" max="27" width="20.7109375" customWidth="1"/>
+    <col min="28" max="28" width="6.7109375" customWidth="1"/>
+    <col min="29" max="29" width="1.7109375" customWidth="1"/>
+    <col min="30" max="30" width="2.7109375" customWidth="1"/>
+    <col min="31" max="31" width="20.7109375" customWidth="1"/>
+    <col min="32" max="32" width="6.7109375" customWidth="1"/>
+    <col min="33" max="33" width="1.7109375" customWidth="1"/>
+    <col min="34" max="34" width="2.7109375" customWidth="1"/>
+    <col min="35" max="35" width="20.7109375" customWidth="1"/>
+    <col min="36" max="36" width="6.7109375" customWidth="1"/>
+    <col min="37" max="37" width="1.7109375" customWidth="1"/>
+    <col min="38" max="38" width="2.7109375" customWidth="1"/>
+    <col min="39" max="39" width="20.7109375" customWidth="1"/>
+    <col min="40" max="40" width="6.7109375" customWidth="1"/>
+    <col min="41" max="41" width="2.7109375" customWidth="1"/>
+    <col min="42" max="42" width="16.7109375" customWidth="1"/>
+    <col min="43" max="43" width="3.7109375" customWidth="1"/>
+    <col min="44" max="44" width="8.28515625" customWidth="1"/>
     <col min="45" max="48" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="12"/>
       <c r="B1" s="111" t="s">
         <v>0</v>
@@ -2172,7 +2178,7 @@
       <c r="AQ1" s="12"/>
       <c r="AR1" s="13"/>
     </row>
-    <row r="2" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
       <c r="B2" s="114">
         <f>N2-3</f>
@@ -2247,7 +2253,7 @@
       <c r="AQ2" s="12"/>
       <c r="AR2" s="13"/>
     </row>
-    <row r="3" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="12"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -2293,7 +2299,7 @@
       <c r="AQ3" s="12"/>
       <c r="AR3" s="13"/>
     </row>
-    <row r="4" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="12"/>
       <c r="B4" s="120"/>
       <c r="C4" s="120"/>
@@ -2341,7 +2347,7 @@
       <c r="AQ4" s="12"/>
       <c r="AR4" s="13"/>
     </row>
-    <row r="5" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="12"/>
       <c r="B5" s="120"/>
       <c r="C5" s="120"/>
@@ -2387,7 +2393,7 @@
       <c r="AQ5" s="12"/>
       <c r="AR5" s="13"/>
     </row>
-    <row r="6" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="75"/>
       <c r="C6" s="76"/>
       <c r="D6" s="59"/>
@@ -2400,32 +2406,32 @@
       <c r="K6" s="76"/>
       <c r="L6" s="59"/>
       <c r="M6" s="3"/>
-      <c r="N6" s="83"/>
-      <c r="O6" s="84"/>
+      <c r="N6" s="86"/>
+      <c r="O6" s="87"/>
       <c r="P6" s="34"/>
       <c r="Q6" s="39"/>
-      <c r="R6" s="83"/>
-      <c r="S6" s="84"/>
+      <c r="R6" s="86"/>
+      <c r="S6" s="87"/>
       <c r="T6" s="34"/>
       <c r="U6" s="36"/>
-      <c r="V6" s="83"/>
-      <c r="W6" s="84"/>
+      <c r="V6" s="86"/>
+      <c r="W6" s="87"/>
       <c r="X6" s="34"/>
       <c r="Y6" s="23"/>
-      <c r="Z6" s="83"/>
-      <c r="AA6" s="84"/>
+      <c r="Z6" s="86"/>
+      <c r="AA6" s="87"/>
       <c r="AB6" s="34"/>
       <c r="AC6" s="36"/>
-      <c r="AD6" s="83"/>
-      <c r="AE6" s="84"/>
+      <c r="AD6" s="86"/>
+      <c r="AE6" s="87"/>
       <c r="AF6" s="34"/>
       <c r="AG6" s="39"/>
-      <c r="AH6" s="83"/>
-      <c r="AI6" s="84"/>
+      <c r="AH6" s="86"/>
+      <c r="AI6" s="87"/>
       <c r="AJ6" s="34"/>
       <c r="AK6" s="36"/>
-      <c r="AL6" s="83"/>
-      <c r="AM6" s="84"/>
+      <c r="AL6" s="86"/>
+      <c r="AM6" s="87"/>
       <c r="AN6" s="34"/>
       <c r="AP6" s="46" t="s">
         <v>7</v>
@@ -2436,7 +2442,7 @@
       </c>
       <c r="AR6" s="30"/>
     </row>
-    <row r="7" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="66"/>
       <c r="C7" s="67"/>
       <c r="D7" s="60"/>
@@ -2485,7 +2491,7 @@
       </c>
       <c r="AR7" s="30"/>
     </row>
-    <row r="8" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="69"/>
       <c r="C8" s="70"/>
       <c r="D8" s="71"/>
@@ -2534,46 +2540,46 @@
       </c>
       <c r="AR8" s="30"/>
     </row>
-    <row r="9" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="88"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="90"/>
+    <row r="9" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="77"/>
+      <c r="C9" s="78"/>
+      <c r="D9" s="79"/>
       <c r="E9" s="43"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="89"/>
-      <c r="H9" s="90"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="78"/>
+      <c r="H9" s="79"/>
       <c r="I9" s="43"/>
-      <c r="J9" s="88"/>
-      <c r="K9" s="89"/>
-      <c r="L9" s="90"/>
+      <c r="J9" s="77"/>
+      <c r="K9" s="78"/>
+      <c r="L9" s="79"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="88"/>
-      <c r="O9" s="89"/>
-      <c r="P9" s="90"/>
+      <c r="N9" s="77"/>
+      <c r="O9" s="78"/>
+      <c r="P9" s="79"/>
       <c r="Q9" s="43"/>
-      <c r="R9" s="88"/>
-      <c r="S9" s="89"/>
-      <c r="T9" s="90"/>
+      <c r="R9" s="77"/>
+      <c r="S9" s="78"/>
+      <c r="T9" s="79"/>
       <c r="U9" s="44"/>
-      <c r="V9" s="88"/>
-      <c r="W9" s="89"/>
-      <c r="X9" s="90"/>
+      <c r="V9" s="77"/>
+      <c r="W9" s="78"/>
+      <c r="X9" s="79"/>
       <c r="Y9" s="43"/>
-      <c r="Z9" s="88"/>
-      <c r="AA9" s="89"/>
-      <c r="AB9" s="90"/>
+      <c r="Z9" s="77"/>
+      <c r="AA9" s="78"/>
+      <c r="AB9" s="79"/>
       <c r="AC9" s="43"/>
-      <c r="AD9" s="88"/>
-      <c r="AE9" s="89"/>
-      <c r="AF9" s="90"/>
+      <c r="AD9" s="77"/>
+      <c r="AE9" s="78"/>
+      <c r="AF9" s="79"/>
       <c r="AG9" s="43"/>
-      <c r="AH9" s="88"/>
-      <c r="AI9" s="89"/>
-      <c r="AJ9" s="90"/>
+      <c r="AH9" s="77"/>
+      <c r="AI9" s="78"/>
+      <c r="AJ9" s="79"/>
       <c r="AK9" s="43"/>
-      <c r="AL9" s="88"/>
-      <c r="AM9" s="89"/>
-      <c r="AN9" s="90"/>
+      <c r="AL9" s="77"/>
+      <c r="AM9" s="78"/>
+      <c r="AN9" s="79"/>
       <c r="AP9" s="46" t="s">
         <v>11</v>
       </c>
@@ -2583,7 +2589,7 @@
       </c>
       <c r="AR9" s="30"/>
     </row>
-    <row r="10" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="107"/>
       <c r="C10" s="108"/>
       <c r="D10" s="109"/>
@@ -2632,7 +2638,7 @@
       </c>
       <c r="AR10" s="30"/>
     </row>
-    <row r="11" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="33"/>
       <c r="C11" s="33"/>
       <c r="D11" s="33"/>
@@ -2681,7 +2687,7 @@
       </c>
       <c r="AR11" s="30"/>
     </row>
-    <row r="12" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="75"/>
       <c r="C12" s="76"/>
       <c r="D12" s="59"/>
@@ -2694,43 +2700,43 @@
       <c r="K12" s="76"/>
       <c r="L12" s="59"/>
       <c r="M12" s="5"/>
-      <c r="N12" s="83"/>
-      <c r="O12" s="84"/>
+      <c r="N12" s="86"/>
+      <c r="O12" s="87"/>
       <c r="P12" s="34"/>
       <c r="Q12" s="23"/>
-      <c r="R12" s="83"/>
-      <c r="S12" s="84"/>
+      <c r="R12" s="86"/>
+      <c r="S12" s="87"/>
       <c r="T12" s="34"/>
       <c r="U12" s="36"/>
-      <c r="V12" s="83"/>
-      <c r="W12" s="84"/>
+      <c r="V12" s="86"/>
+      <c r="W12" s="87"/>
       <c r="X12" s="34"/>
       <c r="Y12" s="23"/>
-      <c r="Z12" s="83"/>
-      <c r="AA12" s="84"/>
+      <c r="Z12" s="86"/>
+      <c r="AA12" s="87"/>
       <c r="AB12" s="34"/>
       <c r="AC12" s="36"/>
-      <c r="AD12" s="83"/>
-      <c r="AE12" s="84"/>
+      <c r="AD12" s="86"/>
+      <c r="AE12" s="87"/>
       <c r="AF12" s="34"/>
       <c r="AG12" s="39"/>
-      <c r="AH12" s="83"/>
-      <c r="AI12" s="84"/>
+      <c r="AH12" s="86"/>
+      <c r="AI12" s="87"/>
       <c r="AJ12" s="34"/>
       <c r="AK12" s="36"/>
-      <c r="AL12" s="83"/>
-      <c r="AM12" s="84"/>
+      <c r="AL12" s="86"/>
+      <c r="AM12" s="87"/>
       <c r="AN12" s="34"/>
       <c r="AP12" s="46" t="s">
         <v>19</v>
       </c>
       <c r="AQ12" s="25">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR12" s="30"/>
     </row>
-    <row r="13" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="66"/>
       <c r="C13" s="67"/>
       <c r="D13" s="60"/>
@@ -2743,17 +2749,17 @@
       <c r="K13" s="64"/>
       <c r="L13" s="65"/>
       <c r="M13" s="5"/>
-      <c r="N13" s="85"/>
-      <c r="O13" s="86"/>
-      <c r="P13" s="87"/>
+      <c r="N13" s="88"/>
+      <c r="O13" s="89"/>
+      <c r="P13" s="90"/>
       <c r="Q13" s="36"/>
-      <c r="R13" s="85"/>
-      <c r="S13" s="86"/>
-      <c r="T13" s="87"/>
+      <c r="R13" s="88"/>
+      <c r="S13" s="89"/>
+      <c r="T13" s="90"/>
       <c r="U13" s="36"/>
-      <c r="V13" s="85"/>
-      <c r="W13" s="86"/>
-      <c r="X13" s="87"/>
+      <c r="V13" s="88"/>
+      <c r="W13" s="89"/>
+      <c r="X13" s="90"/>
       <c r="Y13" s="36"/>
       <c r="Z13" s="91"/>
       <c r="AA13" s="92"/>
@@ -2763,13 +2769,13 @@
       <c r="AE13" s="92"/>
       <c r="AF13" s="18"/>
       <c r="AG13" s="38"/>
-      <c r="AH13" s="85"/>
-      <c r="AI13" s="86"/>
-      <c r="AJ13" s="87"/>
+      <c r="AH13" s="88"/>
+      <c r="AI13" s="89"/>
+      <c r="AJ13" s="90"/>
       <c r="AK13" s="36"/>
-      <c r="AL13" s="85"/>
-      <c r="AM13" s="86"/>
-      <c r="AN13" s="87"/>
+      <c r="AL13" s="88"/>
+      <c r="AM13" s="89"/>
+      <c r="AN13" s="90"/>
       <c r="AP13" s="61" t="s">
         <v>22</v>
       </c>
@@ -2781,7 +2787,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="69"/>
       <c r="C14" s="70"/>
       <c r="D14" s="71"/>
@@ -2832,46 +2838,46 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="88"/>
-      <c r="C15" s="89"/>
-      <c r="D15" s="90"/>
+    <row r="15" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="77"/>
+      <c r="C15" s="78"/>
+      <c r="D15" s="79"/>
       <c r="E15" s="44"/>
-      <c r="F15" s="88"/>
-      <c r="G15" s="89"/>
-      <c r="H15" s="90"/>
+      <c r="F15" s="77"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="79"/>
       <c r="I15" s="43"/>
-      <c r="J15" s="88"/>
-      <c r="K15" s="89"/>
-      <c r="L15" s="90"/>
+      <c r="J15" s="77"/>
+      <c r="K15" s="78"/>
+      <c r="L15" s="79"/>
       <c r="M15" s="3"/>
-      <c r="N15" s="88"/>
-      <c r="O15" s="89"/>
-      <c r="P15" s="90"/>
+      <c r="N15" s="77"/>
+      <c r="O15" s="78"/>
+      <c r="P15" s="79"/>
       <c r="Q15" s="43"/>
-      <c r="R15" s="88"/>
-      <c r="S15" s="89"/>
-      <c r="T15" s="90"/>
+      <c r="R15" s="77"/>
+      <c r="S15" s="78"/>
+      <c r="T15" s="79"/>
       <c r="U15" s="44"/>
-      <c r="V15" s="88"/>
-      <c r="W15" s="89"/>
-      <c r="X15" s="90"/>
+      <c r="V15" s="77"/>
+      <c r="W15" s="78"/>
+      <c r="X15" s="79"/>
       <c r="Y15" s="43"/>
-      <c r="Z15" s="88"/>
-      <c r="AA15" s="89"/>
-      <c r="AB15" s="90"/>
+      <c r="Z15" s="77"/>
+      <c r="AA15" s="78"/>
+      <c r="AB15" s="79"/>
       <c r="AC15" s="43"/>
-      <c r="AD15" s="88"/>
-      <c r="AE15" s="89"/>
-      <c r="AF15" s="90"/>
+      <c r="AD15" s="77"/>
+      <c r="AE15" s="78"/>
+      <c r="AF15" s="79"/>
       <c r="AG15" s="44"/>
-      <c r="AH15" s="88"/>
-      <c r="AI15" s="89"/>
-      <c r="AJ15" s="90"/>
+      <c r="AH15" s="77"/>
+      <c r="AI15" s="78"/>
+      <c r="AJ15" s="79"/>
       <c r="AK15" s="43"/>
-      <c r="AL15" s="88"/>
-      <c r="AM15" s="89"/>
-      <c r="AN15" s="90"/>
+      <c r="AL15" s="77"/>
+      <c r="AM15" s="78"/>
+      <c r="AN15" s="79"/>
       <c r="AP15" s="46" t="s">
         <v>18</v>
       </c>
@@ -2881,7 +2887,7 @@
       </c>
       <c r="AR15" s="30"/>
     </row>
-    <row r="16" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B16" s="107"/>
       <c r="C16" s="108"/>
       <c r="D16" s="109"/>
@@ -2926,11 +2932,11 @@
       </c>
       <c r="AQ16" s="25">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR16" s="30"/>
     </row>
-    <row r="17" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="33"/>
       <c r="C17" s="33"/>
       <c r="D17" s="33"/>
@@ -2979,7 +2985,7 @@
       </c>
       <c r="AR17" s="30"/>
     </row>
-    <row r="18" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="33"/>
       <c r="C18" s="33"/>
       <c r="D18" s="33"/>
@@ -3030,7 +3036,7 @@
       </c>
       <c r="AR18" s="30"/>
     </row>
-    <row r="19" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="33"/>
       <c r="C19" s="33"/>
       <c r="D19" s="33"/>
@@ -3079,7 +3085,7 @@
       </c>
       <c r="AR19" s="30"/>
     </row>
-    <row r="20" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="75"/>
       <c r="C20" s="76"/>
       <c r="D20" s="59"/>
@@ -3092,8 +3098,8 @@
       <c r="K20" s="76"/>
       <c r="L20" s="59"/>
       <c r="M20" s="4"/>
-      <c r="N20" s="83"/>
-      <c r="O20" s="84"/>
+      <c r="N20" s="86"/>
+      <c r="O20" s="87"/>
       <c r="P20" s="34"/>
       <c r="Q20" s="36"/>
       <c r="R20" s="125"/>
@@ -3108,16 +3114,16 @@
       <c r="AA20" s="126"/>
       <c r="AB20" s="56"/>
       <c r="AC20" s="36"/>
-      <c r="AD20" s="83"/>
-      <c r="AE20" s="84"/>
+      <c r="AD20" s="86"/>
+      <c r="AE20" s="87"/>
       <c r="AF20" s="34"/>
       <c r="AG20" s="36"/>
-      <c r="AH20" s="83"/>
-      <c r="AI20" s="84"/>
+      <c r="AH20" s="86"/>
+      <c r="AI20" s="87"/>
       <c r="AJ20" s="34"/>
       <c r="AK20" s="36"/>
-      <c r="AL20" s="83"/>
-      <c r="AM20" s="84"/>
+      <c r="AL20" s="86"/>
+      <c r="AM20" s="87"/>
       <c r="AN20" s="34"/>
       <c r="AP20" s="46" t="s">
         <v>26</v>
@@ -3128,7 +3134,7 @@
       </c>
       <c r="AR20" s="30"/>
     </row>
-    <row r="21" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="66"/>
       <c r="C21" s="67"/>
       <c r="D21" s="60"/>
@@ -3177,17 +3183,17 @@
       </c>
       <c r="AR21" s="30"/>
     </row>
-    <row r="22" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="77"/>
-      <c r="C22" s="78"/>
+    <row r="22" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="80"/>
+      <c r="C22" s="81"/>
       <c r="D22" s="41"/>
       <c r="E22" s="37"/>
-      <c r="F22" s="77"/>
-      <c r="G22" s="78"/>
+      <c r="F22" s="80"/>
+      <c r="G22" s="81"/>
       <c r="H22" s="41"/>
       <c r="I22" s="35"/>
-      <c r="J22" s="77"/>
-      <c r="K22" s="78"/>
+      <c r="J22" s="80"/>
+      <c r="K22" s="81"/>
       <c r="L22" s="41"/>
       <c r="M22" s="4"/>
       <c r="N22" s="94"/>
@@ -3206,12 +3212,12 @@
       <c r="AA22" s="95"/>
       <c r="AB22" s="58"/>
       <c r="AC22" s="35"/>
-      <c r="AD22" s="77"/>
-      <c r="AE22" s="78"/>
+      <c r="AD22" s="80"/>
+      <c r="AE22" s="81"/>
       <c r="AF22" s="41"/>
       <c r="AG22" s="37"/>
-      <c r="AH22" s="77"/>
-      <c r="AI22" s="78"/>
+      <c r="AH22" s="80"/>
+      <c r="AI22" s="81"/>
       <c r="AJ22" s="41"/>
       <c r="AK22" s="35"/>
       <c r="AL22" s="94"/>
@@ -3226,7 +3232,7 @@
       </c>
       <c r="AR22" s="30"/>
     </row>
-    <row r="23" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="96"/>
       <c r="C23" s="97"/>
       <c r="D23" s="45"/>
@@ -3271,98 +3277,98 @@
       </c>
       <c r="AQ23" s="25">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR23" s="30"/>
     </row>
-    <row r="24" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="81"/>
-      <c r="C24" s="82"/>
+    <row r="24" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="84"/>
+      <c r="C24" s="85"/>
       <c r="D24" s="45"/>
       <c r="E24" s="43"/>
-      <c r="F24" s="81"/>
-      <c r="G24" s="82"/>
+      <c r="F24" s="84"/>
+      <c r="G24" s="85"/>
       <c r="H24" s="45"/>
       <c r="I24" s="44"/>
-      <c r="J24" s="81"/>
-      <c r="K24" s="82"/>
+      <c r="J24" s="84"/>
+      <c r="K24" s="85"/>
       <c r="L24" s="45"/>
       <c r="M24" s="14"/>
-      <c r="N24" s="81"/>
-      <c r="O24" s="82"/>
+      <c r="N24" s="84"/>
+      <c r="O24" s="85"/>
       <c r="P24" s="45"/>
       <c r="Q24" s="43"/>
-      <c r="R24" s="81"/>
-      <c r="S24" s="82"/>
+      <c r="R24" s="84"/>
+      <c r="S24" s="85"/>
       <c r="T24" s="45"/>
       <c r="U24" s="44"/>
-      <c r="V24" s="81"/>
-      <c r="W24" s="82"/>
+      <c r="V24" s="84"/>
+      <c r="W24" s="85"/>
       <c r="X24" s="45"/>
       <c r="Y24" s="43"/>
-      <c r="Z24" s="81"/>
-      <c r="AA24" s="82"/>
+      <c r="Z24" s="84"/>
+      <c r="AA24" s="85"/>
       <c r="AB24" s="45"/>
       <c r="AC24" s="43"/>
-      <c r="AD24" s="81"/>
-      <c r="AE24" s="82"/>
+      <c r="AD24" s="84"/>
+      <c r="AE24" s="85"/>
       <c r="AF24" s="45"/>
       <c r="AG24" s="43"/>
-      <c r="AH24" s="81"/>
-      <c r="AI24" s="82"/>
+      <c r="AH24" s="84"/>
+      <c r="AI24" s="85"/>
       <c r="AJ24" s="45"/>
       <c r="AK24" s="44"/>
-      <c r="AL24" s="81"/>
-      <c r="AM24" s="82"/>
+      <c r="AL24" s="84"/>
+      <c r="AM24" s="85"/>
       <c r="AN24" s="45"/>
       <c r="AP24" s="46" t="s">
         <v>14</v>
       </c>
       <c r="AQ24" s="25">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR24" s="30"/>
     </row>
-    <row r="25" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="81"/>
-      <c r="C25" s="82"/>
+    <row r="25" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="84"/>
+      <c r="C25" s="85"/>
       <c r="D25" s="45"/>
       <c r="E25" s="44"/>
-      <c r="F25" s="81"/>
-      <c r="G25" s="82"/>
+      <c r="F25" s="84"/>
+      <c r="G25" s="85"/>
       <c r="H25" s="45"/>
       <c r="I25" s="44"/>
-      <c r="J25" s="81"/>
-      <c r="K25" s="82"/>
+      <c r="J25" s="84"/>
+      <c r="K25" s="85"/>
       <c r="L25" s="45"/>
       <c r="M25" s="4"/>
-      <c r="N25" s="81"/>
-      <c r="O25" s="82"/>
+      <c r="N25" s="84"/>
+      <c r="O25" s="85"/>
       <c r="P25" s="45"/>
       <c r="Q25" s="44"/>
-      <c r="R25" s="81"/>
-      <c r="S25" s="82"/>
+      <c r="R25" s="84"/>
+      <c r="S25" s="85"/>
       <c r="T25" s="45"/>
       <c r="U25" s="44"/>
-      <c r="V25" s="81"/>
-      <c r="W25" s="82"/>
+      <c r="V25" s="84"/>
+      <c r="W25" s="85"/>
       <c r="X25" s="45"/>
       <c r="Y25" s="44"/>
-      <c r="Z25" s="81"/>
-      <c r="AA25" s="82"/>
+      <c r="Z25" s="84"/>
+      <c r="AA25" s="85"/>
       <c r="AB25" s="45"/>
       <c r="AC25" s="44"/>
-      <c r="AD25" s="81"/>
-      <c r="AE25" s="82"/>
+      <c r="AD25" s="84"/>
+      <c r="AE25" s="85"/>
       <c r="AF25" s="45"/>
       <c r="AG25" s="44"/>
-      <c r="AH25" s="81"/>
-      <c r="AI25" s="82"/>
+      <c r="AH25" s="84"/>
+      <c r="AI25" s="85"/>
       <c r="AJ25" s="45"/>
       <c r="AK25" s="44"/>
-      <c r="AL25" s="81"/>
-      <c r="AM25" s="82"/>
+      <c r="AL25" s="84"/>
+      <c r="AM25" s="85"/>
       <c r="AN25" s="45"/>
       <c r="AP25" s="46" t="s">
         <v>21</v>
@@ -3373,94 +3379,94 @@
       </c>
       <c r="AR25" s="30"/>
     </row>
-    <row r="26" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="81"/>
-      <c r="C26" s="82"/>
+    <row r="26" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="84"/>
+      <c r="C26" s="85"/>
       <c r="D26" s="45"/>
       <c r="E26" s="44"/>
-      <c r="F26" s="81"/>
-      <c r="G26" s="82"/>
+      <c r="F26" s="84"/>
+      <c r="G26" s="85"/>
       <c r="H26" s="45"/>
       <c r="I26" s="44"/>
-      <c r="J26" s="81"/>
-      <c r="K26" s="82"/>
+      <c r="J26" s="84"/>
+      <c r="K26" s="85"/>
       <c r="L26" s="45"/>
       <c r="M26" s="4"/>
-      <c r="N26" s="81"/>
-      <c r="O26" s="82"/>
+      <c r="N26" s="84"/>
+      <c r="O26" s="85"/>
       <c r="P26" s="45"/>
       <c r="Q26" s="44"/>
-      <c r="R26" s="81"/>
-      <c r="S26" s="82"/>
+      <c r="R26" s="84"/>
+      <c r="S26" s="85"/>
       <c r="T26" s="45"/>
       <c r="U26" s="44"/>
-      <c r="V26" s="81"/>
-      <c r="W26" s="82"/>
+      <c r="V26" s="84"/>
+      <c r="W26" s="85"/>
       <c r="X26" s="45"/>
       <c r="Y26" s="44"/>
-      <c r="Z26" s="81"/>
-      <c r="AA26" s="82"/>
+      <c r="Z26" s="84"/>
+      <c r="AA26" s="85"/>
       <c r="AB26" s="45"/>
       <c r="AC26" s="44"/>
-      <c r="AD26" s="81"/>
-      <c r="AE26" s="82"/>
+      <c r="AD26" s="84"/>
+      <c r="AE26" s="85"/>
       <c r="AF26" s="45"/>
       <c r="AG26" s="44"/>
-      <c r="AH26" s="81"/>
-      <c r="AI26" s="82"/>
+      <c r="AH26" s="84"/>
+      <c r="AI26" s="85"/>
       <c r="AJ26" s="45"/>
       <c r="AK26" s="44"/>
-      <c r="AL26" s="81"/>
-      <c r="AM26" s="82"/>
+      <c r="AL26" s="84"/>
+      <c r="AM26" s="85"/>
       <c r="AN26" s="45"/>
       <c r="AP26" s="46" t="s">
         <v>27</v>
       </c>
       <c r="AQ26" s="25">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AR26" s="30"/>
     </row>
-    <row r="27" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="79"/>
-      <c r="C27" s="80"/>
+    <row r="27" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="82"/>
+      <c r="C27" s="83"/>
       <c r="D27" s="42"/>
       <c r="E27" s="44"/>
-      <c r="F27" s="79"/>
-      <c r="G27" s="80"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="83"/>
       <c r="H27" s="42"/>
       <c r="I27" s="44"/>
-      <c r="J27" s="79"/>
-      <c r="K27" s="80"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="83"/>
       <c r="L27" s="42"/>
       <c r="M27" s="5"/>
-      <c r="N27" s="79"/>
-      <c r="O27" s="80"/>
+      <c r="N27" s="82"/>
+      <c r="O27" s="83"/>
       <c r="P27" s="42"/>
       <c r="Q27" s="44"/>
-      <c r="R27" s="79"/>
-      <c r="S27" s="80"/>
+      <c r="R27" s="82"/>
+      <c r="S27" s="83"/>
       <c r="T27" s="42"/>
       <c r="U27" s="44"/>
-      <c r="V27" s="79"/>
-      <c r="W27" s="80"/>
+      <c r="V27" s="82"/>
+      <c r="W27" s="83"/>
       <c r="X27" s="42"/>
       <c r="Y27" s="44"/>
-      <c r="Z27" s="79"/>
-      <c r="AA27" s="80"/>
+      <c r="Z27" s="82"/>
+      <c r="AA27" s="83"/>
       <c r="AB27" s="42"/>
       <c r="AC27" s="44"/>
-      <c r="AD27" s="79"/>
-      <c r="AE27" s="80"/>
+      <c r="AD27" s="82"/>
+      <c r="AE27" s="83"/>
       <c r="AF27" s="42"/>
       <c r="AG27" s="44"/>
-      <c r="AH27" s="79"/>
-      <c r="AI27" s="80"/>
+      <c r="AH27" s="82"/>
+      <c r="AI27" s="83"/>
       <c r="AJ27" s="42"/>
       <c r="AK27" s="44"/>
-      <c r="AL27" s="79"/>
-      <c r="AM27" s="80"/>
+      <c r="AL27" s="82"/>
+      <c r="AM27" s="83"/>
       <c r="AN27" s="42"/>
       <c r="AP27" s="46" t="s">
         <v>13</v>
@@ -3471,7 +3477,7 @@
       </c>
       <c r="AR27" s="30"/>
     </row>
-    <row r="28" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="33"/>
       <c r="C28" s="33"/>
       <c r="D28" s="33"/>
@@ -3520,7 +3526,7 @@
       </c>
       <c r="AR28" s="30"/>
     </row>
-    <row r="29" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="33"/>
       <c r="C29" s="33"/>
       <c r="D29" s="33"/>
@@ -3571,7 +3577,7 @@
       </c>
       <c r="AR29" s="30"/>
     </row>
-    <row r="30" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B30" s="33"/>
       <c r="C30" s="33"/>
       <c r="D30" s="33"/>
@@ -3620,7 +3626,7 @@
       </c>
       <c r="AR30" s="30"/>
     </row>
-    <row r="31" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="75" t="s">
         <v>45</v>
       </c>
@@ -3639,52 +3645,50 @@
       <c r="K31" s="76"/>
       <c r="L31" s="59"/>
       <c r="M31" s="6"/>
-      <c r="N31" s="83" t="s">
+      <c r="N31" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="O31" s="84"/>
+      <c r="O31" s="87"/>
       <c r="P31" s="34"/>
       <c r="Q31" s="36"/>
-      <c r="R31" s="83" t="s">
+      <c r="R31" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="S31" s="84"/>
+      <c r="S31" s="87"/>
       <c r="T31" s="34"/>
       <c r="U31" s="36"/>
-      <c r="V31" s="83" t="s">
+      <c r="V31" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="W31" s="84"/>
+      <c r="W31" s="87"/>
       <c r="X31" s="34"/>
       <c r="Y31" s="36"/>
-      <c r="Z31" s="83" t="s">
+      <c r="Z31" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="AA31" s="84"/>
+      <c r="AA31" s="87"/>
       <c r="AB31" s="34"/>
       <c r="AC31" s="36"/>
-      <c r="AD31" s="101" t="s">
-        <v>69</v>
-      </c>
-      <c r="AE31" s="102"/>
+      <c r="AD31" s="104" t="s">
+        <v>54</v>
+      </c>
+      <c r="AE31" s="105"/>
       <c r="AF31" s="62"/>
       <c r="AG31" s="36"/>
-      <c r="AH31" s="83" t="s">
-        <v>54</v>
-      </c>
-      <c r="AI31" s="84"/>
+      <c r="AH31" s="86"/>
+      <c r="AI31" s="87"/>
       <c r="AJ31" s="34"/>
       <c r="AK31" s="36"/>
-      <c r="AL31" s="83" t="s">
+      <c r="AL31" s="86" t="s">
         <v>54</v>
       </c>
-      <c r="AM31" s="84"/>
+      <c r="AM31" s="87"/>
       <c r="AN31" s="34"/>
       <c r="AP31" s="48"/>
       <c r="AQ31" s="49"/>
       <c r="AR31" s="30"/>
     </row>
-    <row r="32" spans="2:44" s="16" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:44" s="16" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B32" s="63" t="s">
         <v>46</v>
       </c>
@@ -3703,52 +3707,50 @@
       <c r="K32" s="64"/>
       <c r="L32" s="65"/>
       <c r="M32" s="5"/>
-      <c r="N32" s="85" t="s">
+      <c r="N32" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="O32" s="86"/>
-      <c r="P32" s="87"/>
+      <c r="O32" s="89"/>
+      <c r="P32" s="90"/>
       <c r="Q32" s="36"/>
-      <c r="R32" s="85" t="s">
+      <c r="R32" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="S32" s="86"/>
-      <c r="T32" s="87"/>
+      <c r="S32" s="89"/>
+      <c r="T32" s="90"/>
       <c r="U32" s="36"/>
-      <c r="V32" s="85" t="s">
+      <c r="V32" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="W32" s="86"/>
-      <c r="X32" s="87"/>
+      <c r="W32" s="89"/>
+      <c r="X32" s="90"/>
       <c r="Y32" s="37"/>
-      <c r="Z32" s="85" t="s">
+      <c r="Z32" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="AA32" s="86"/>
-      <c r="AB32" s="87"/>
+      <c r="AA32" s="89"/>
+      <c r="AB32" s="90"/>
       <c r="AC32" s="36"/>
       <c r="AD32" s="98" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AE32" s="99"/>
       <c r="AF32" s="100"/>
       <c r="AG32" s="36"/>
-      <c r="AH32" s="85" t="s">
+      <c r="AH32" s="88"/>
+      <c r="AI32" s="89"/>
+      <c r="AJ32" s="90"/>
+      <c r="AK32" s="36"/>
+      <c r="AL32" s="88" t="s">
         <v>55</v>
       </c>
-      <c r="AI32" s="86"/>
-      <c r="AJ32" s="87"/>
-      <c r="AK32" s="36"/>
-      <c r="AL32" s="85" t="s">
-        <v>55</v>
-      </c>
-      <c r="AM32" s="86"/>
-      <c r="AN32" s="87"/>
+      <c r="AM32" s="89"/>
+      <c r="AN32" s="90"/>
       <c r="AP32" s="51"/>
       <c r="AQ32" s="52"/>
       <c r="AR32" s="30"/>
     </row>
-    <row r="33" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="66" t="s">
         <v>47</v>
       </c>
@@ -3791,24 +3793,24 @@
       <c r="AA33" s="92"/>
       <c r="AB33" s="93"/>
       <c r="AC33" s="36"/>
-      <c r="AD33" s="103"/>
-      <c r="AE33" s="104"/>
-      <c r="AF33" s="105"/>
+      <c r="AD33" s="101" t="s">
+        <v>70</v>
+      </c>
+      <c r="AE33" s="102"/>
+      <c r="AF33" s="103"/>
       <c r="AG33" s="43"/>
-      <c r="AH33" s="91" t="s">
-        <v>58</v>
-      </c>
+      <c r="AH33" s="91"/>
       <c r="AI33" s="92"/>
       <c r="AJ33" s="93"/>
       <c r="AK33" s="32"/>
       <c r="AL33" s="91" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="AM33" s="92"/>
       <c r="AN33" s="93"/>
       <c r="AR33" s="13"/>
     </row>
-    <row r="34" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="12"/>
       <c r="B34" s="69" t="s">
         <v>7</v>
@@ -3853,14 +3855,12 @@
       <c r="AB34" s="71"/>
       <c r="AC34" s="32"/>
       <c r="AD34" s="69" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="AE34" s="70"/>
       <c r="AF34" s="71"/>
       <c r="AG34" s="37"/>
-      <c r="AH34" s="69" t="s">
-        <v>24</v>
-      </c>
+      <c r="AH34" s="69"/>
       <c r="AI34" s="70"/>
       <c r="AJ34" s="71"/>
       <c r="AK34" s="35"/>
@@ -3874,7 +3874,7 @@
       <c r="AQ34" s="12"/>
       <c r="AR34" s="13"/>
     </row>
-    <row r="35" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="12"/>
       <c r="B35" s="72" t="s">
         <v>17</v>
@@ -3918,28 +3918,26 @@
       <c r="AA35" s="73"/>
       <c r="AB35" s="74"/>
       <c r="AC35" s="32"/>
-      <c r="AD35" s="88" t="s">
-        <v>13</v>
-      </c>
-      <c r="AE35" s="89"/>
-      <c r="AF35" s="90"/>
+      <c r="AD35" s="77" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE35" s="78"/>
+      <c r="AF35" s="79"/>
       <c r="AG35" s="44"/>
-      <c r="AH35" s="88" t="s">
+      <c r="AH35" s="77"/>
+      <c r="AI35" s="78"/>
+      <c r="AJ35" s="79"/>
+      <c r="AK35" s="44"/>
+      <c r="AL35" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="AI35" s="89"/>
-      <c r="AJ35" s="90"/>
-      <c r="AK35" s="44"/>
-      <c r="AL35" s="88" t="s">
-        <v>19</v>
-      </c>
-      <c r="AM35" s="89"/>
-      <c r="AN35" s="90"/>
+      <c r="AM35" s="78"/>
+      <c r="AN35" s="79"/>
       <c r="AO35" s="12"/>
       <c r="AQ35" s="12"/>
       <c r="AR35" s="13"/>
     </row>
-    <row r="36" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="12"/>
       <c r="B36" s="35"/>
       <c r="C36" s="35"/>
@@ -3973,9 +3971,7 @@
       <c r="AE36" s="73"/>
       <c r="AF36" s="74"/>
       <c r="AG36" s="35"/>
-      <c r="AH36" s="72" t="s">
-        <v>27</v>
-      </c>
+      <c r="AH36" s="72"/>
       <c r="AI36" s="73"/>
       <c r="AJ36" s="74"/>
       <c r="AK36" s="35"/>
@@ -3989,7 +3985,7 @@
       <c r="AQ36" s="31"/>
       <c r="AR36" s="13"/>
     </row>
-    <row r="37" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="12"/>
       <c r="B37" s="75" t="s">
         <v>45</v>
@@ -4009,28 +4005,28 @@
       <c r="K37" s="76"/>
       <c r="L37" s="59"/>
       <c r="M37" s="5"/>
-      <c r="N37" s="83" t="s">
+      <c r="N37" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="O37" s="84"/>
+      <c r="O37" s="87"/>
       <c r="P37" s="34"/>
       <c r="Q37" s="36"/>
-      <c r="R37" s="83" t="s">
+      <c r="R37" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="S37" s="84"/>
+      <c r="S37" s="87"/>
       <c r="T37" s="34"/>
       <c r="U37" s="50"/>
-      <c r="V37" s="83" t="s">
+      <c r="V37" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="W37" s="84"/>
+      <c r="W37" s="87"/>
       <c r="X37" s="34"/>
       <c r="Y37" s="32"/>
-      <c r="Z37" s="83" t="s">
+      <c r="Z37" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="AA37" s="84"/>
+      <c r="AA37" s="87"/>
       <c r="AB37" s="34"/>
       <c r="AC37" s="36"/>
       <c r="AD37" s="35"/>
@@ -4049,7 +4045,7 @@
       <c r="AQ37" s="31"/>
       <c r="AR37" s="13"/>
     </row>
-    <row r="38" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="12"/>
       <c r="B38" s="63" t="s">
         <v>46</v>
@@ -4069,51 +4065,51 @@
       <c r="K38" s="64"/>
       <c r="L38" s="65"/>
       <c r="M38" s="5"/>
-      <c r="N38" s="85" t="s">
+      <c r="N38" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="O38" s="86"/>
-      <c r="P38" s="87"/>
+      <c r="O38" s="89"/>
+      <c r="P38" s="90"/>
       <c r="Q38" s="36"/>
-      <c r="R38" s="85" t="s">
+      <c r="R38" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="S38" s="86"/>
-      <c r="T38" s="87"/>
+      <c r="S38" s="89"/>
+      <c r="T38" s="90"/>
       <c r="U38" s="32"/>
-      <c r="V38" s="85" t="s">
+      <c r="V38" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="W38" s="86"/>
-      <c r="X38" s="87"/>
+      <c r="W38" s="89"/>
+      <c r="X38" s="90"/>
       <c r="Y38" s="54"/>
-      <c r="Z38" s="85" t="s">
+      <c r="Z38" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="AA38" s="86"/>
-      <c r="AB38" s="87"/>
+      <c r="AA38" s="89"/>
+      <c r="AB38" s="90"/>
       <c r="AC38" s="36"/>
-      <c r="AD38" s="83"/>
-      <c r="AE38" s="84"/>
+      <c r="AD38" s="86"/>
+      <c r="AE38" s="87"/>
       <c r="AF38" s="34"/>
       <c r="AG38" s="36"/>
-      <c r="AH38" s="101" t="s">
+      <c r="AH38" s="104" t="s">
         <v>57</v>
       </c>
-      <c r="AI38" s="102"/>
+      <c r="AI38" s="105"/>
       <c r="AJ38" s="62"/>
       <c r="AK38" s="36"/>
-      <c r="AL38" s="83" t="s">
+      <c r="AL38" s="86" t="s">
         <v>57</v>
       </c>
-      <c r="AM38" s="84"/>
+      <c r="AM38" s="87"/>
       <c r="AN38" s="34"/>
       <c r="AO38" s="31"/>
       <c r="AP38" s="31"/>
       <c r="AQ38" s="31"/>
       <c r="AR38" s="13"/>
     </row>
-    <row r="39" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="12"/>
       <c r="B39" s="66" t="s">
         <v>48</v>
@@ -4157,9 +4153,9 @@
       <c r="AA39" s="92"/>
       <c r="AB39" s="93"/>
       <c r="AC39" s="36"/>
-      <c r="AD39" s="85"/>
-      <c r="AE39" s="86"/>
-      <c r="AF39" s="87"/>
+      <c r="AD39" s="88"/>
+      <c r="AE39" s="89"/>
+      <c r="AF39" s="90"/>
       <c r="AG39" s="36"/>
       <c r="AH39" s="98" t="s">
         <v>59</v>
@@ -4167,17 +4163,17 @@
       <c r="AI39" s="99"/>
       <c r="AJ39" s="100"/>
       <c r="AK39" s="36"/>
-      <c r="AL39" s="85" t="s">
+      <c r="AL39" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="AM39" s="86"/>
-      <c r="AN39" s="87"/>
+      <c r="AM39" s="89"/>
+      <c r="AN39" s="90"/>
       <c r="AO39" s="31"/>
       <c r="AP39" s="31"/>
       <c r="AQ39" s="31"/>
       <c r="AR39" s="13"/>
     </row>
-    <row r="40" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="12"/>
       <c r="B40" s="69" t="s">
         <v>9</v>
@@ -4225,11 +4221,11 @@
       <c r="AE40" s="92"/>
       <c r="AF40" s="93"/>
       <c r="AG40" s="43"/>
-      <c r="AH40" s="103" t="s">
+      <c r="AH40" s="101" t="s">
         <v>58</v>
       </c>
-      <c r="AI40" s="104"/>
-      <c r="AJ40" s="105"/>
+      <c r="AI40" s="102"/>
+      <c r="AJ40" s="103"/>
       <c r="AK40" s="32"/>
       <c r="AL40" s="91"/>
       <c r="AM40" s="92"/>
@@ -4239,7 +4235,7 @@
       <c r="AQ40" s="31"/>
       <c r="AR40" s="13"/>
     </row>
-    <row r="41" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="12"/>
       <c r="B41" s="72" t="s">
         <v>8</v>
@@ -4303,7 +4299,7 @@
       <c r="AQ41" s="31"/>
       <c r="AR41" s="13"/>
     </row>
-    <row r="42" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="12"/>
       <c r="B42" s="35"/>
       <c r="C42" s="35"/>
@@ -4333,27 +4329,27 @@
       <c r="AA42" s="35"/>
       <c r="AB42" s="35"/>
       <c r="AC42" s="35"/>
-      <c r="AD42" s="88"/>
-      <c r="AE42" s="89"/>
-      <c r="AF42" s="90"/>
+      <c r="AD42" s="77"/>
+      <c r="AE42" s="78"/>
+      <c r="AF42" s="79"/>
       <c r="AG42" s="35"/>
-      <c r="AH42" s="88" t="s">
+      <c r="AH42" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="AI42" s="89"/>
-      <c r="AJ42" s="90"/>
+      <c r="AI42" s="78"/>
+      <c r="AJ42" s="79"/>
       <c r="AK42" s="35"/>
-      <c r="AL42" s="88" t="s">
+      <c r="AL42" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="AM42" s="89"/>
-      <c r="AN42" s="90"/>
+      <c r="AM42" s="78"/>
+      <c r="AN42" s="79"/>
       <c r="AO42" s="31"/>
       <c r="AP42" s="31"/>
       <c r="AQ42" s="31"/>
       <c r="AR42" s="13"/>
     </row>
-    <row r="43" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="12"/>
       <c r="B43" s="75" t="s">
         <v>45</v>
@@ -4373,28 +4369,28 @@
       <c r="K43" s="76"/>
       <c r="L43" s="59"/>
       <c r="M43" s="14"/>
-      <c r="N43" s="83" t="s">
+      <c r="N43" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="O43" s="84"/>
+      <c r="O43" s="87"/>
       <c r="P43" s="34"/>
       <c r="Q43" s="50"/>
-      <c r="R43" s="83" t="s">
+      <c r="R43" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="S43" s="84"/>
+      <c r="S43" s="87"/>
       <c r="T43" s="34"/>
       <c r="U43" s="50"/>
-      <c r="V43" s="83" t="s">
+      <c r="V43" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="W43" s="84"/>
+      <c r="W43" s="87"/>
       <c r="X43" s="34"/>
       <c r="Y43" s="50"/>
-      <c r="Z43" s="83" t="s">
+      <c r="Z43" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="AA43" s="84"/>
+      <c r="AA43" s="87"/>
       <c r="AB43" s="34"/>
       <c r="AC43" s="50"/>
       <c r="AD43" s="72"/>
@@ -4417,7 +4413,7 @@
       <c r="AQ43" s="31"/>
       <c r="AR43" s="13"/>
     </row>
-    <row r="44" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="12"/>
       <c r="B44" s="63" t="s">
         <v>46</v>
@@ -4437,29 +4433,29 @@
       <c r="K44" s="64"/>
       <c r="L44" s="65"/>
       <c r="M44" s="14"/>
-      <c r="N44" s="85" t="s">
+      <c r="N44" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="O44" s="86"/>
-      <c r="P44" s="87"/>
+      <c r="O44" s="89"/>
+      <c r="P44" s="90"/>
       <c r="Q44" s="35"/>
-      <c r="R44" s="85" t="s">
+      <c r="R44" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="S44" s="86"/>
-      <c r="T44" s="87"/>
+      <c r="S44" s="89"/>
+      <c r="T44" s="90"/>
       <c r="U44" s="36"/>
-      <c r="V44" s="85" t="s">
+      <c r="V44" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="W44" s="86"/>
-      <c r="X44" s="87"/>
+      <c r="W44" s="89"/>
+      <c r="X44" s="90"/>
       <c r="Y44" s="36"/>
-      <c r="Z44" s="85" t="s">
+      <c r="Z44" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="AA44" s="86"/>
-      <c r="AB44" s="87"/>
+      <c r="AA44" s="89"/>
+      <c r="AB44" s="90"/>
       <c r="AC44" s="36"/>
       <c r="AD44" s="35"/>
       <c r="AE44" s="35"/>
@@ -4477,7 +4473,7 @@
       <c r="AQ44" s="31"/>
       <c r="AR44" s="13"/>
     </row>
-    <row r="45" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12"/>
       <c r="B45" s="66" t="s">
         <v>49</v>
@@ -4521,18 +4517,20 @@
       <c r="AA45" s="92"/>
       <c r="AB45" s="93"/>
       <c r="AC45" s="36"/>
-      <c r="AD45" s="83"/>
-      <c r="AE45" s="84"/>
+      <c r="AD45" s="86"/>
+      <c r="AE45" s="87"/>
       <c r="AF45" s="34"/>
       <c r="AG45" s="36"/>
-      <c r="AH45" s="83"/>
-      <c r="AI45" s="84"/>
-      <c r="AJ45" s="34"/>
+      <c r="AH45" s="104" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI45" s="105"/>
+      <c r="AJ45" s="62"/>
       <c r="AK45" s="50"/>
-      <c r="AL45" s="83" t="s">
+      <c r="AL45" s="86" t="s">
         <v>44</v>
       </c>
-      <c r="AM45" s="84"/>
+      <c r="AM45" s="87"/>
       <c r="AN45" s="34" t="s">
         <v>43</v>
       </c>
@@ -4541,119 +4539,121 @@
       <c r="AQ45" s="31"/>
       <c r="AR45" s="13"/>
     </row>
-    <row r="46" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12"/>
-      <c r="B46" s="88" t="s">
+      <c r="B46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="C46" s="89"/>
-      <c r="D46" s="90"/>
+      <c r="C46" s="78"/>
+      <c r="D46" s="79"/>
       <c r="E46" s="36"/>
-      <c r="F46" s="88" t="s">
+      <c r="F46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="G46" s="89"/>
-      <c r="H46" s="90"/>
+      <c r="G46" s="78"/>
+      <c r="H46" s="79"/>
       <c r="I46" s="32"/>
-      <c r="J46" s="88" t="s">
+      <c r="J46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="K46" s="89"/>
-      <c r="L46" s="90"/>
+      <c r="K46" s="78"/>
+      <c r="L46" s="79"/>
       <c r="M46" s="4"/>
-      <c r="N46" s="88" t="s">
+      <c r="N46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="O46" s="89"/>
-      <c r="P46" s="90"/>
+      <c r="O46" s="78"/>
+      <c r="P46" s="79"/>
       <c r="Q46" s="32"/>
-      <c r="R46" s="88" t="s">
+      <c r="R46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="S46" s="89"/>
-      <c r="T46" s="90"/>
+      <c r="S46" s="78"/>
+      <c r="T46" s="79"/>
       <c r="U46" s="36"/>
-      <c r="V46" s="88" t="s">
+      <c r="V46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="W46" s="89"/>
-      <c r="X46" s="90"/>
+      <c r="W46" s="78"/>
+      <c r="X46" s="79"/>
       <c r="Y46" s="36"/>
-      <c r="Z46" s="88" t="s">
+      <c r="Z46" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="AA46" s="89"/>
-      <c r="AB46" s="90"/>
+      <c r="AA46" s="78"/>
+      <c r="AB46" s="79"/>
       <c r="AC46" s="35"/>
-      <c r="AD46" s="85"/>
-      <c r="AE46" s="86"/>
-      <c r="AF46" s="87"/>
+      <c r="AD46" s="88"/>
+      <c r="AE46" s="89"/>
+      <c r="AF46" s="90"/>
       <c r="AG46" s="36"/>
-      <c r="AH46" s="85"/>
-      <c r="AI46" s="86"/>
-      <c r="AJ46" s="87"/>
+      <c r="AH46" s="98" t="s">
+        <v>69</v>
+      </c>
+      <c r="AI46" s="99"/>
+      <c r="AJ46" s="100"/>
       <c r="AK46" s="32"/>
-      <c r="AL46" s="85" t="s">
+      <c r="AL46" s="88" t="s">
         <v>56</v>
       </c>
-      <c r="AM46" s="86"/>
-      <c r="AN46" s="87"/>
+      <c r="AM46" s="89"/>
+      <c r="AN46" s="90"/>
       <c r="AO46" s="31"/>
       <c r="AP46" s="31"/>
       <c r="AQ46" s="31"/>
       <c r="AR46" s="13"/>
     </row>
-    <row r="47" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12"/>
-      <c r="B47" s="88" t="s">
+      <c r="B47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="C47" s="89"/>
-      <c r="D47" s="90"/>
+      <c r="C47" s="78"/>
+      <c r="D47" s="79"/>
       <c r="E47" s="43"/>
-      <c r="F47" s="88" t="s">
+      <c r="F47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="G47" s="89"/>
-      <c r="H47" s="90"/>
+      <c r="G47" s="78"/>
+      <c r="H47" s="79"/>
       <c r="I47" s="32"/>
-      <c r="J47" s="88" t="s">
+      <c r="J47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="K47" s="89"/>
-      <c r="L47" s="90"/>
+      <c r="K47" s="78"/>
+      <c r="L47" s="79"/>
       <c r="M47" s="4"/>
-      <c r="N47" s="88" t="s">
+      <c r="N47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="O47" s="89"/>
-      <c r="P47" s="90"/>
+      <c r="O47" s="78"/>
+      <c r="P47" s="79"/>
       <c r="Q47" s="43"/>
-      <c r="R47" s="88" t="s">
+      <c r="R47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="S47" s="89"/>
-      <c r="T47" s="90"/>
+      <c r="S47" s="78"/>
+      <c r="T47" s="79"/>
       <c r="U47" s="32"/>
-      <c r="V47" s="88" t="s">
+      <c r="V47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="W47" s="89"/>
-      <c r="X47" s="90"/>
+      <c r="W47" s="78"/>
+      <c r="X47" s="79"/>
       <c r="Y47" s="32"/>
-      <c r="Z47" s="88" t="s">
+      <c r="Z47" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="AA47" s="89"/>
-      <c r="AB47" s="90"/>
+      <c r="AA47" s="78"/>
+      <c r="AB47" s="79"/>
       <c r="AC47" s="31"/>
       <c r="AD47" s="91"/>
       <c r="AE47" s="92"/>
       <c r="AF47" s="93"/>
       <c r="AG47" s="43"/>
-      <c r="AH47" s="91"/>
-      <c r="AI47" s="92"/>
-      <c r="AJ47" s="93"/>
+      <c r="AH47" s="101"/>
+      <c r="AI47" s="102"/>
+      <c r="AJ47" s="103"/>
       <c r="AK47" s="32"/>
       <c r="AL47" s="91"/>
       <c r="AM47" s="92"/>
@@ -4663,57 +4663,59 @@
       <c r="AQ47" s="31"/>
       <c r="AR47" s="13"/>
     </row>
-    <row r="48" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12"/>
-      <c r="B48" s="88" t="s">
+      <c r="B48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="C48" s="89"/>
-      <c r="D48" s="90"/>
+      <c r="C48" s="78"/>
+      <c r="D48" s="79"/>
       <c r="E48" s="37"/>
-      <c r="F48" s="88" t="s">
+      <c r="F48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="G48" s="89"/>
-      <c r="H48" s="90"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="79"/>
       <c r="I48" s="37"/>
-      <c r="J48" s="88" t="s">
+      <c r="J48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="K48" s="89"/>
-      <c r="L48" s="90"/>
+      <c r="K48" s="78"/>
+      <c r="L48" s="79"/>
       <c r="M48" s="5"/>
-      <c r="N48" s="88" t="s">
+      <c r="N48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="O48" s="89"/>
-      <c r="P48" s="90"/>
+      <c r="O48" s="78"/>
+      <c r="P48" s="79"/>
       <c r="Q48" s="43"/>
-      <c r="R48" s="88" t="s">
+      <c r="R48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="S48" s="89"/>
-      <c r="T48" s="90"/>
+      <c r="S48" s="78"/>
+      <c r="T48" s="79"/>
       <c r="U48" s="35"/>
-      <c r="V48" s="88" t="s">
+      <c r="V48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="W48" s="89"/>
-      <c r="X48" s="90"/>
+      <c r="W48" s="78"/>
+      <c r="X48" s="79"/>
       <c r="Y48" s="35"/>
-      <c r="Z48" s="88" t="s">
+      <c r="Z48" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="AA48" s="89"/>
-      <c r="AB48" s="90"/>
+      <c r="AA48" s="78"/>
+      <c r="AB48" s="79"/>
       <c r="AC48" s="35"/>
-      <c r="AD48" s="88"/>
-      <c r="AE48" s="89"/>
-      <c r="AF48" s="90"/>
+      <c r="AD48" s="77"/>
+      <c r="AE48" s="78"/>
+      <c r="AF48" s="79"/>
       <c r="AG48" s="37"/>
-      <c r="AH48" s="88"/>
-      <c r="AI48" s="89"/>
-      <c r="AJ48" s="90"/>
+      <c r="AH48" s="69" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI48" s="70"/>
+      <c r="AJ48" s="71"/>
       <c r="AK48" s="37"/>
       <c r="AL48" s="69" t="s">
         <v>16</v>
@@ -4725,7 +4727,7 @@
       <c r="AQ48" s="31"/>
       <c r="AR48" s="13"/>
     </row>
-    <row r="49" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B49" s="72" t="s">
         <v>26</v>
       </c>
@@ -4768,25 +4770,27 @@
       <c r="AA49" s="73"/>
       <c r="AB49" s="74"/>
       <c r="AC49" s="44"/>
-      <c r="AD49" s="88"/>
-      <c r="AE49" s="89"/>
-      <c r="AF49" s="90"/>
+      <c r="AD49" s="77"/>
+      <c r="AE49" s="78"/>
+      <c r="AF49" s="79"/>
       <c r="AG49" s="44"/>
-      <c r="AH49" s="88"/>
-      <c r="AI49" s="89"/>
-      <c r="AJ49" s="90"/>
+      <c r="AH49" s="77" t="s">
+        <v>13</v>
+      </c>
+      <c r="AI49" s="78"/>
+      <c r="AJ49" s="79"/>
       <c r="AK49" s="44"/>
-      <c r="AL49" s="88" t="s">
+      <c r="AL49" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="AM49" s="89"/>
-      <c r="AN49" s="90"/>
+      <c r="AM49" s="78"/>
+      <c r="AN49" s="79"/>
       <c r="AO49" s="31"/>
       <c r="AP49" s="31"/>
       <c r="AQ49" s="31"/>
       <c r="AR49" s="13"/>
     </row>
-    <row r="50" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B50" s="35"/>
       <c r="C50" s="35"/>
       <c r="D50" s="35"/>
@@ -4831,7 +4835,7 @@
       <c r="AQ50" s="31"/>
       <c r="AR50" s="13"/>
     </row>
-    <row r="51" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="75" t="s">
         <v>45</v>
       </c>
@@ -4850,28 +4854,28 @@
       <c r="K51" s="76"/>
       <c r="L51" s="59"/>
       <c r="M51" s="14"/>
-      <c r="N51" s="83" t="s">
+      <c r="N51" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="O51" s="84"/>
+      <c r="O51" s="87"/>
       <c r="P51" s="34"/>
       <c r="Q51" s="40"/>
-      <c r="R51" s="83" t="s">
+      <c r="R51" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="S51" s="84"/>
+      <c r="S51" s="87"/>
       <c r="T51" s="34"/>
       <c r="U51" s="40"/>
-      <c r="V51" s="83" t="s">
+      <c r="V51" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="W51" s="84"/>
+      <c r="W51" s="87"/>
       <c r="X51" s="34"/>
       <c r="Y51" s="32"/>
-      <c r="Z51" s="83" t="s">
+      <c r="Z51" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="AA51" s="84"/>
+      <c r="AA51" s="87"/>
       <c r="AB51" s="34"/>
       <c r="AC51" s="40"/>
       <c r="AD51" s="35"/>
@@ -4890,7 +4894,7 @@
       <c r="AQ51" s="31"/>
       <c r="AR51" s="13"/>
     </row>
-    <row r="52" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="63" t="s">
         <v>46</v>
       </c>
@@ -4909,44 +4913,44 @@
       <c r="K52" s="64"/>
       <c r="L52" s="65"/>
       <c r="M52" s="14"/>
-      <c r="N52" s="85" t="s">
+      <c r="N52" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="O52" s="86"/>
-      <c r="P52" s="87"/>
+      <c r="O52" s="89"/>
+      <c r="P52" s="90"/>
       <c r="Q52" s="36"/>
-      <c r="R52" s="85" t="s">
+      <c r="R52" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="S52" s="86"/>
-      <c r="T52" s="87"/>
+      <c r="S52" s="89"/>
+      <c r="T52" s="90"/>
       <c r="U52" s="32"/>
-      <c r="V52" s="85" t="s">
+      <c r="V52" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="W52" s="86"/>
-      <c r="X52" s="87"/>
+      <c r="W52" s="89"/>
+      <c r="X52" s="90"/>
       <c r="Y52" s="54"/>
-      <c r="Z52" s="85" t="s">
+      <c r="Z52" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="AA52" s="86"/>
-      <c r="AB52" s="87"/>
+      <c r="AA52" s="89"/>
+      <c r="AB52" s="90"/>
       <c r="AC52" s="36"/>
-      <c r="AD52" s="83"/>
-      <c r="AE52" s="84"/>
+      <c r="AD52" s="86"/>
+      <c r="AE52" s="87"/>
       <c r="AF52" s="34"/>
       <c r="AG52" s="50"/>
-      <c r="AH52" s="83"/>
-      <c r="AI52" s="84"/>
+      <c r="AH52" s="86"/>
+      <c r="AI52" s="87"/>
       <c r="AJ52" s="34"/>
       <c r="AK52" s="32"/>
-      <c r="AL52" s="83"/>
-      <c r="AM52" s="84"/>
+      <c r="AL52" s="86"/>
+      <c r="AM52" s="87"/>
       <c r="AN52" s="34"/>
       <c r="AR52" s="13"/>
     </row>
-    <row r="53" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="66" t="s">
         <v>50</v>
       </c>
@@ -4989,20 +4993,20 @@
       <c r="AA53" s="92"/>
       <c r="AB53" s="93"/>
       <c r="AC53" s="36"/>
-      <c r="AD53" s="85"/>
-      <c r="AE53" s="86"/>
-      <c r="AF53" s="87"/>
+      <c r="AD53" s="88"/>
+      <c r="AE53" s="89"/>
+      <c r="AF53" s="90"/>
       <c r="AG53" s="32"/>
-      <c r="AH53" s="85"/>
-      <c r="AI53" s="86"/>
-      <c r="AJ53" s="87"/>
+      <c r="AH53" s="88"/>
+      <c r="AI53" s="89"/>
+      <c r="AJ53" s="90"/>
       <c r="AK53" s="54"/>
-      <c r="AL53" s="85"/>
-      <c r="AM53" s="86"/>
-      <c r="AN53" s="87"/>
+      <c r="AL53" s="88"/>
+      <c r="AM53" s="89"/>
+      <c r="AN53" s="90"/>
       <c r="AR53" s="13"/>
     </row>
-    <row r="54" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="69" t="s">
         <v>24</v>
       </c>
@@ -5058,48 +5062,48 @@
       <c r="AN54" s="93"/>
       <c r="AR54" s="13"/>
     </row>
-    <row r="55" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="88" t="s">
+    <row r="55" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="C55" s="89"/>
-      <c r="D55" s="90"/>
+      <c r="C55" s="78"/>
+      <c r="D55" s="79"/>
       <c r="E55" s="37"/>
-      <c r="F55" s="88" t="s">
+      <c r="F55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="G55" s="89"/>
-      <c r="H55" s="90"/>
+      <c r="G55" s="78"/>
+      <c r="H55" s="79"/>
       <c r="I55" s="35"/>
-      <c r="J55" s="88" t="s">
+      <c r="J55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="K55" s="89"/>
-      <c r="L55" s="90"/>
+      <c r="K55" s="78"/>
+      <c r="L55" s="79"/>
       <c r="M55" s="5"/>
-      <c r="N55" s="88" t="s">
+      <c r="N55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="O55" s="89"/>
-      <c r="P55" s="90"/>
+      <c r="O55" s="78"/>
+      <c r="P55" s="79"/>
       <c r="Q55" s="44"/>
-      <c r="R55" s="88" t="s">
+      <c r="R55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="S55" s="89"/>
-      <c r="T55" s="90"/>
+      <c r="S55" s="78"/>
+      <c r="T55" s="79"/>
       <c r="U55" s="44"/>
-      <c r="V55" s="88" t="s">
+      <c r="V55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="W55" s="89"/>
-      <c r="X55" s="90"/>
+      <c r="W55" s="78"/>
+      <c r="X55" s="79"/>
       <c r="Y55" s="40"/>
-      <c r="Z55" s="88" t="s">
+      <c r="Z55" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="AA55" s="89"/>
-      <c r="AB55" s="90"/>
+      <c r="AA55" s="78"/>
+      <c r="AB55" s="79"/>
       <c r="AC55" s="43"/>
       <c r="AD55" s="69"/>
       <c r="AE55" s="70"/>
@@ -5114,7 +5118,7 @@
       <c r="AN55" s="71"/>
       <c r="AR55" s="13"/>
     </row>
-    <row r="56" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B56" s="72" t="s">
         <v>21</v>
       </c>
@@ -5157,20 +5161,20 @@
       <c r="AA56" s="73"/>
       <c r="AB56" s="74"/>
       <c r="AC56" s="44"/>
-      <c r="AD56" s="88"/>
-      <c r="AE56" s="89"/>
-      <c r="AF56" s="90"/>
+      <c r="AD56" s="77"/>
+      <c r="AE56" s="78"/>
+      <c r="AF56" s="79"/>
       <c r="AG56" s="44"/>
-      <c r="AH56" s="88"/>
-      <c r="AI56" s="89"/>
-      <c r="AJ56" s="90"/>
+      <c r="AH56" s="77"/>
+      <c r="AI56" s="78"/>
+      <c r="AJ56" s="79"/>
       <c r="AK56" s="40"/>
-      <c r="AL56" s="88"/>
-      <c r="AM56" s="89"/>
-      <c r="AN56" s="90"/>
+      <c r="AL56" s="77"/>
+      <c r="AM56" s="78"/>
+      <c r="AN56" s="79"/>
       <c r="AR56" s="13"/>
     </row>
-    <row r="57" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B57" s="35"/>
       <c r="C57" s="35"/>
       <c r="D57" s="35"/>
@@ -5212,7 +5216,7 @@
       <c r="AN57" s="74"/>
       <c r="AR57" s="13"/>
     </row>
-    <row r="58" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="127" t="s">
         <v>45</v>
       </c>
@@ -5229,28 +5233,28 @@
       <c r="K58" s="76"/>
       <c r="L58" s="59"/>
       <c r="M58" s="5"/>
-      <c r="N58" s="83" t="s">
+      <c r="N58" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="O58" s="84"/>
+      <c r="O58" s="87"/>
       <c r="P58" s="34"/>
       <c r="Q58" s="31"/>
-      <c r="R58" s="83" t="s">
+      <c r="R58" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="S58" s="84"/>
+      <c r="S58" s="87"/>
       <c r="T58" s="34"/>
       <c r="U58" s="50"/>
-      <c r="V58" s="83" t="s">
+      <c r="V58" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="W58" s="84"/>
+      <c r="W58" s="87"/>
       <c r="X58" s="34"/>
       <c r="Y58" s="35"/>
-      <c r="Z58" s="83" t="s">
+      <c r="Z58" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="AA58" s="84"/>
+      <c r="AA58" s="87"/>
       <c r="AB58" s="34"/>
       <c r="AC58" s="50"/>
       <c r="AD58" s="35"/>
@@ -5266,7 +5270,7 @@
       <c r="AN58" s="35"/>
       <c r="AR58" s="13"/>
     </row>
-    <row r="59" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="63" t="s">
         <v>46</v>
       </c>
@@ -5283,44 +5287,44 @@
       <c r="K59" s="64"/>
       <c r="L59" s="65"/>
       <c r="M59" s="6"/>
-      <c r="N59" s="85" t="s">
+      <c r="N59" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="O59" s="86"/>
-      <c r="P59" s="87"/>
+      <c r="O59" s="89"/>
+      <c r="P59" s="90"/>
       <c r="Q59" s="36"/>
-      <c r="R59" s="85" t="s">
+      <c r="R59" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="S59" s="86"/>
-      <c r="T59" s="87"/>
+      <c r="S59" s="89"/>
+      <c r="T59" s="90"/>
       <c r="U59" s="32"/>
-      <c r="V59" s="85" t="s">
+      <c r="V59" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="W59" s="86"/>
-      <c r="X59" s="87"/>
+      <c r="W59" s="89"/>
+      <c r="X59" s="90"/>
       <c r="Y59" s="54"/>
-      <c r="Z59" s="85" t="s">
+      <c r="Z59" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="AA59" s="86"/>
-      <c r="AB59" s="87"/>
+      <c r="AA59" s="89"/>
+      <c r="AB59" s="90"/>
       <c r="AC59" s="36"/>
-      <c r="AD59" s="83"/>
-      <c r="AE59" s="84"/>
+      <c r="AD59" s="86"/>
+      <c r="AE59" s="87"/>
       <c r="AF59" s="34"/>
       <c r="AG59" s="36"/>
-      <c r="AH59" s="83"/>
-      <c r="AI59" s="84"/>
+      <c r="AH59" s="86"/>
+      <c r="AI59" s="87"/>
       <c r="AJ59" s="34"/>
       <c r="AK59" s="32"/>
-      <c r="AL59" s="83"/>
-      <c r="AM59" s="84"/>
+      <c r="AL59" s="86"/>
+      <c r="AM59" s="87"/>
       <c r="AN59" s="34"/>
       <c r="AR59" s="13"/>
     </row>
-    <row r="60" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="66" t="s">
         <v>61</v>
       </c>
@@ -5361,20 +5365,20 @@
       <c r="AA60" s="92"/>
       <c r="AB60" s="93"/>
       <c r="AC60" s="36"/>
-      <c r="AD60" s="85"/>
-      <c r="AE60" s="86"/>
-      <c r="AF60" s="87"/>
+      <c r="AD60" s="88"/>
+      <c r="AE60" s="89"/>
+      <c r="AF60" s="90"/>
       <c r="AG60" s="36"/>
-      <c r="AH60" s="85"/>
-      <c r="AI60" s="86"/>
-      <c r="AJ60" s="87"/>
+      <c r="AH60" s="88"/>
+      <c r="AI60" s="89"/>
+      <c r="AJ60" s="90"/>
       <c r="AK60" s="54"/>
-      <c r="AL60" s="85"/>
-      <c r="AM60" s="86"/>
-      <c r="AN60" s="87"/>
+      <c r="AL60" s="88"/>
+      <c r="AM60" s="89"/>
+      <c r="AN60" s="90"/>
       <c r="AR60" s="13"/>
     </row>
-    <row r="61" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="69" t="s">
         <v>18</v>
       </c>
@@ -5428,103 +5432,103 @@
       <c r="AN61" s="93"/>
       <c r="AR61" s="13"/>
     </row>
-    <row r="62" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="88" t="s">
+    <row r="62" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="C62" s="89"/>
-      <c r="D62" s="90"/>
+      <c r="C62" s="78"/>
+      <c r="D62" s="79"/>
       <c r="E62" s="37"/>
-      <c r="F62" s="88"/>
-      <c r="G62" s="89"/>
-      <c r="H62" s="90"/>
+      <c r="F62" s="77"/>
+      <c r="G62" s="78"/>
+      <c r="H62" s="79"/>
       <c r="I62" s="37"/>
-      <c r="J62" s="88" t="s">
+      <c r="J62" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="K62" s="89"/>
-      <c r="L62" s="90"/>
+      <c r="K62" s="78"/>
+      <c r="L62" s="79"/>
       <c r="M62" s="4"/>
-      <c r="N62" s="88" t="s">
+      <c r="N62" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="O62" s="89"/>
-      <c r="P62" s="90"/>
+      <c r="O62" s="78"/>
+      <c r="P62" s="79"/>
       <c r="Q62" s="44"/>
-      <c r="R62" s="88" t="s">
+      <c r="R62" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="S62" s="89"/>
-      <c r="T62" s="90"/>
+      <c r="S62" s="78"/>
+      <c r="T62" s="79"/>
       <c r="U62" s="44"/>
-      <c r="V62" s="88" t="s">
+      <c r="V62" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="W62" s="89"/>
-      <c r="X62" s="90"/>
+      <c r="W62" s="78"/>
+      <c r="X62" s="79"/>
       <c r="Y62" s="40"/>
-      <c r="Z62" s="88" t="s">
+      <c r="Z62" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="AA62" s="89"/>
-      <c r="AB62" s="90"/>
+      <c r="AA62" s="78"/>
+      <c r="AB62" s="79"/>
       <c r="AC62" s="43"/>
-      <c r="AD62" s="88"/>
-      <c r="AE62" s="89"/>
-      <c r="AF62" s="90"/>
+      <c r="AD62" s="77"/>
+      <c r="AE62" s="78"/>
+      <c r="AF62" s="79"/>
       <c r="AG62" s="37"/>
-      <c r="AH62" s="88"/>
-      <c r="AI62" s="89"/>
-      <c r="AJ62" s="90"/>
+      <c r="AH62" s="77"/>
+      <c r="AI62" s="78"/>
+      <c r="AJ62" s="79"/>
       <c r="AK62" s="37"/>
-      <c r="AL62" s="88"/>
-      <c r="AM62" s="89"/>
-      <c r="AN62" s="90"/>
+      <c r="AL62" s="77"/>
+      <c r="AM62" s="78"/>
+      <c r="AN62" s="79"/>
       <c r="AR62" s="13"/>
     </row>
-    <row r="63" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="88"/>
-      <c r="C63" s="89"/>
-      <c r="D63" s="90"/>
+    <row r="63" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B63" s="77"/>
+      <c r="C63" s="78"/>
+      <c r="D63" s="79"/>
       <c r="E63" s="44"/>
-      <c r="F63" s="88"/>
-      <c r="G63" s="89"/>
-      <c r="H63" s="90"/>
+      <c r="F63" s="77"/>
+      <c r="G63" s="78"/>
+      <c r="H63" s="79"/>
       <c r="I63" s="44"/>
-      <c r="J63" s="88"/>
-      <c r="K63" s="89"/>
-      <c r="L63" s="90"/>
+      <c r="J63" s="77"/>
+      <c r="K63" s="78"/>
+      <c r="L63" s="79"/>
       <c r="M63" s="5"/>
-      <c r="N63" s="88"/>
-      <c r="O63" s="89"/>
-      <c r="P63" s="90"/>
+      <c r="N63" s="77"/>
+      <c r="O63" s="78"/>
+      <c r="P63" s="79"/>
       <c r="Q63" s="44"/>
-      <c r="R63" s="88"/>
-      <c r="S63" s="89"/>
-      <c r="T63" s="90"/>
+      <c r="R63" s="77"/>
+      <c r="S63" s="78"/>
+      <c r="T63" s="79"/>
       <c r="U63" s="44"/>
-      <c r="V63" s="88"/>
-      <c r="W63" s="89"/>
-      <c r="X63" s="90"/>
+      <c r="V63" s="77"/>
+      <c r="W63" s="78"/>
+      <c r="X63" s="79"/>
       <c r="Y63" s="50"/>
-      <c r="Z63" s="88"/>
-      <c r="AA63" s="89"/>
-      <c r="AB63" s="90"/>
+      <c r="Z63" s="77"/>
+      <c r="AA63" s="78"/>
+      <c r="AB63" s="79"/>
       <c r="AC63" s="44"/>
-      <c r="AD63" s="88"/>
-      <c r="AE63" s="89"/>
-      <c r="AF63" s="90"/>
+      <c r="AD63" s="77"/>
+      <c r="AE63" s="78"/>
+      <c r="AF63" s="79"/>
       <c r="AG63" s="44"/>
-      <c r="AH63" s="88"/>
-      <c r="AI63" s="89"/>
-      <c r="AJ63" s="90"/>
+      <c r="AH63" s="77"/>
+      <c r="AI63" s="78"/>
+      <c r="AJ63" s="79"/>
       <c r="AK63" s="44"/>
-      <c r="AL63" s="88"/>
-      <c r="AM63" s="89"/>
-      <c r="AN63" s="90"/>
+      <c r="AL63" s="77"/>
+      <c r="AM63" s="78"/>
+      <c r="AN63" s="79"/>
       <c r="AR63" s="13"/>
     </row>
-    <row r="64" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:44" s="12" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B64" s="72"/>
       <c r="C64" s="73"/>
       <c r="D64" s="74"/>
@@ -5566,7 +5570,7 @@
       <c r="AN64" s="74"/>
       <c r="AR64" s="13"/>
     </row>
-    <row r="65" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="12"/>
       <c r="B65" s="33"/>
       <c r="C65" s="33"/>
@@ -5612,7 +5616,7 @@
       <c r="AQ65" s="12"/>
       <c r="AR65" s="13"/>
     </row>
-    <row r="66" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="12"/>
       <c r="B66" s="40"/>
       <c r="C66" s="33"/>
@@ -5659,7 +5663,7 @@
       <c r="AQ66" s="12"/>
       <c r="AR66" s="13"/>
     </row>
-    <row r="67" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="12"/>
       <c r="B67" s="33"/>
       <c r="C67" s="33"/>
@@ -5705,7 +5709,7 @@
       <c r="AQ67" s="12"/>
       <c r="AR67" s="13"/>
     </row>
-    <row r="68" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="12"/>
       <c r="B68" s="127" t="s">
         <v>45</v>
@@ -5713,46 +5717,46 @@
       <c r="C68" s="128"/>
       <c r="D68" s="55"/>
       <c r="E68" s="32"/>
-      <c r="F68" s="101" t="s">
+      <c r="F68" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="G68" s="102"/>
+      <c r="G68" s="105"/>
       <c r="H68" s="62"/>
       <c r="I68" s="32"/>
-      <c r="J68" s="101" t="s">
+      <c r="J68" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="K68" s="102"/>
+      <c r="K68" s="105"/>
       <c r="L68" s="62"/>
       <c r="M68" s="4"/>
-      <c r="N68" s="83"/>
-      <c r="O68" s="84"/>
+      <c r="N68" s="86"/>
+      <c r="O68" s="87"/>
       <c r="P68" s="34"/>
       <c r="Q68" s="32"/>
-      <c r="R68" s="83" t="s">
+      <c r="R68" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="S68" s="84"/>
+      <c r="S68" s="87"/>
       <c r="T68" s="34"/>
       <c r="U68" s="36"/>
-      <c r="V68" s="83"/>
-      <c r="W68" s="84"/>
+      <c r="V68" s="86"/>
+      <c r="W68" s="87"/>
       <c r="X68" s="34"/>
       <c r="Y68" s="32"/>
-      <c r="Z68" s="83"/>
-      <c r="AA68" s="84"/>
+      <c r="Z68" s="86"/>
+      <c r="AA68" s="87"/>
       <c r="AB68" s="34"/>
       <c r="AC68" s="32"/>
-      <c r="AD68" s="83"/>
-      <c r="AE68" s="84"/>
+      <c r="AD68" s="86"/>
+      <c r="AE68" s="87"/>
       <c r="AF68" s="34"/>
       <c r="AG68" s="32"/>
-      <c r="AH68" s="83"/>
-      <c r="AI68" s="84"/>
+      <c r="AH68" s="86"/>
+      <c r="AI68" s="87"/>
       <c r="AJ68" s="34"/>
       <c r="AK68" s="32"/>
-      <c r="AL68" s="83"/>
-      <c r="AM68" s="84"/>
+      <c r="AL68" s="86"/>
+      <c r="AM68" s="87"/>
       <c r="AN68" s="34"/>
       <c r="AO68" s="17"/>
       <c r="AP68" s="27" t="s">
@@ -5761,7 +5765,7 @@
       <c r="AQ68" s="12"/>
       <c r="AR68" s="13"/>
     </row>
-    <row r="69" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="12"/>
       <c r="B69" s="63" t="s">
         <v>46</v>
@@ -5781,35 +5785,35 @@
       <c r="K69" s="99"/>
       <c r="L69" s="100"/>
       <c r="M69" s="4"/>
-      <c r="N69" s="85"/>
-      <c r="O69" s="86"/>
-      <c r="P69" s="87"/>
+      <c r="N69" s="88"/>
+      <c r="O69" s="89"/>
+      <c r="P69" s="90"/>
       <c r="Q69" s="35"/>
-      <c r="R69" s="85" t="s">
+      <c r="R69" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="S69" s="86"/>
-      <c r="T69" s="87"/>
+      <c r="S69" s="89"/>
+      <c r="T69" s="90"/>
       <c r="U69" s="32"/>
-      <c r="V69" s="85"/>
-      <c r="W69" s="86"/>
-      <c r="X69" s="87"/>
+      <c r="V69" s="88"/>
+      <c r="W69" s="89"/>
+      <c r="X69" s="90"/>
       <c r="Y69" s="32"/>
-      <c r="Z69" s="85"/>
-      <c r="AA69" s="86"/>
-      <c r="AB69" s="87"/>
+      <c r="Z69" s="88"/>
+      <c r="AA69" s="89"/>
+      <c r="AB69" s="90"/>
       <c r="AC69" s="35"/>
-      <c r="AD69" s="85"/>
-      <c r="AE69" s="86"/>
-      <c r="AF69" s="87"/>
+      <c r="AD69" s="88"/>
+      <c r="AE69" s="89"/>
+      <c r="AF69" s="90"/>
       <c r="AG69" s="32"/>
-      <c r="AH69" s="85"/>
-      <c r="AI69" s="86"/>
-      <c r="AJ69" s="87"/>
+      <c r="AH69" s="88"/>
+      <c r="AI69" s="89"/>
+      <c r="AJ69" s="90"/>
       <c r="AK69" s="32"/>
-      <c r="AL69" s="85"/>
-      <c r="AM69" s="86"/>
-      <c r="AN69" s="87"/>
+      <c r="AL69" s="88"/>
+      <c r="AM69" s="89"/>
+      <c r="AN69" s="90"/>
       <c r="AO69" s="12"/>
       <c r="AP69" s="27" t="s">
         <v>33</v>
@@ -5817,23 +5821,23 @@
       <c r="AQ69" s="12"/>
       <c r="AR69" s="13"/>
     </row>
-    <row r="70" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="12"/>
       <c r="B70" s="66" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C70" s="67"/>
       <c r="D70" s="68"/>
       <c r="E70" s="32"/>
-      <c r="F70" s="103"/>
-      <c r="G70" s="104"/>
-      <c r="H70" s="105"/>
+      <c r="F70" s="101"/>
+      <c r="G70" s="102"/>
+      <c r="H70" s="103"/>
       <c r="I70" s="32"/>
-      <c r="J70" s="103" t="s">
+      <c r="J70" s="101" t="s">
         <v>51</v>
       </c>
-      <c r="K70" s="104"/>
-      <c r="L70" s="105"/>
+      <c r="K70" s="102"/>
+      <c r="L70" s="103"/>
       <c r="M70" s="9"/>
       <c r="N70" s="91"/>
       <c r="O70" s="92"/>
@@ -5871,7 +5875,7 @@
       <c r="AQ70" s="12"/>
       <c r="AR70" s="13"/>
     </row>
-    <row r="71" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="12"/>
       <c r="B71" s="69" t="s">
         <v>64</v>
@@ -5886,7 +5890,7 @@
       <c r="H71" s="71"/>
       <c r="I71" s="32"/>
       <c r="J71" s="129" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="K71" s="130"/>
       <c r="L71" s="131"/>
@@ -5927,7 +5931,7 @@
       <c r="AQ71" s="12"/>
       <c r="AR71" s="13"/>
     </row>
-    <row r="72" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="12"/>
       <c r="B72" s="72" t="s">
         <v>65</v>
@@ -5979,7 +5983,7 @@
       <c r="AQ72" s="12"/>
       <c r="AR72" s="13"/>
     </row>
-    <row r="73" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="12"/>
       <c r="B73" s="35"/>
       <c r="C73" s="35"/>
@@ -6025,7 +6029,7 @@
       <c r="AQ73" s="12"/>
       <c r="AR73" s="13"/>
     </row>
-    <row r="74" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="12"/>
       <c r="B74" s="75" t="s">
         <v>62</v>
@@ -6045,45 +6049,45 @@
       <c r="K74" s="128"/>
       <c r="L74" s="55"/>
       <c r="M74" s="14"/>
-      <c r="N74" s="83"/>
-      <c r="O74" s="84"/>
+      <c r="N74" s="86"/>
+      <c r="O74" s="87"/>
       <c r="P74" s="34"/>
       <c r="Q74" s="44"/>
-      <c r="R74" s="83" t="s">
+      <c r="R74" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="S74" s="84"/>
+      <c r="S74" s="87"/>
       <c r="T74" s="34"/>
       <c r="U74" s="36"/>
-      <c r="V74" s="83"/>
-      <c r="W74" s="84"/>
+      <c r="V74" s="86"/>
+      <c r="W74" s="87"/>
       <c r="X74" s="34"/>
       <c r="Y74" s="32"/>
-      <c r="Z74" s="83" t="s">
+      <c r="Z74" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="AA74" s="84"/>
+      <c r="AA74" s="87"/>
       <c r="AB74" s="34"/>
       <c r="AC74" s="36"/>
-      <c r="AD74" s="83"/>
-      <c r="AE74" s="84"/>
+      <c r="AD74" s="86"/>
+      <c r="AE74" s="87"/>
       <c r="AF74" s="34"/>
       <c r="AG74" s="32"/>
-      <c r="AH74" s="83" t="s">
+      <c r="AH74" s="86" t="s">
         <v>62</v>
       </c>
-      <c r="AI74" s="84"/>
+      <c r="AI74" s="87"/>
       <c r="AJ74" s="34"/>
       <c r="AK74" s="32"/>
-      <c r="AL74" s="83"/>
-      <c r="AM74" s="84"/>
+      <c r="AL74" s="86"/>
+      <c r="AM74" s="87"/>
       <c r="AN74" s="34"/>
       <c r="AO74" s="16"/>
       <c r="AP74" s="28"/>
       <c r="AQ74" s="12"/>
       <c r="AR74" s="13"/>
     </row>
-    <row r="75" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="12"/>
       <c r="B75" s="63"/>
       <c r="C75" s="64"/>
@@ -6097,39 +6101,39 @@
       <c r="K75" s="64"/>
       <c r="L75" s="65"/>
       <c r="M75" s="14"/>
-      <c r="N75" s="85"/>
-      <c r="O75" s="86"/>
-      <c r="P75" s="87"/>
+      <c r="N75" s="88"/>
+      <c r="O75" s="89"/>
+      <c r="P75" s="90"/>
       <c r="Q75" s="44"/>
-      <c r="R75" s="85"/>
-      <c r="S75" s="86"/>
-      <c r="T75" s="87"/>
+      <c r="R75" s="88"/>
+      <c r="S75" s="89"/>
+      <c r="T75" s="90"/>
       <c r="U75" s="32"/>
-      <c r="V75" s="85"/>
-      <c r="W75" s="86"/>
-      <c r="X75" s="87"/>
+      <c r="V75" s="88"/>
+      <c r="W75" s="89"/>
+      <c r="X75" s="90"/>
       <c r="Y75" s="32"/>
-      <c r="Z75" s="85"/>
-      <c r="AA75" s="86"/>
-      <c r="AB75" s="87"/>
+      <c r="Z75" s="88"/>
+      <c r="AA75" s="89"/>
+      <c r="AB75" s="90"/>
       <c r="AC75" s="36"/>
-      <c r="AD75" s="85"/>
-      <c r="AE75" s="86"/>
-      <c r="AF75" s="87"/>
+      <c r="AD75" s="88"/>
+      <c r="AE75" s="89"/>
+      <c r="AF75" s="90"/>
       <c r="AG75" s="32"/>
-      <c r="AH75" s="85"/>
-      <c r="AI75" s="86"/>
-      <c r="AJ75" s="87"/>
+      <c r="AH75" s="88"/>
+      <c r="AI75" s="89"/>
+      <c r="AJ75" s="90"/>
       <c r="AK75" s="32"/>
-      <c r="AL75" s="85"/>
-      <c r="AM75" s="86"/>
-      <c r="AN75" s="87"/>
+      <c r="AL75" s="88"/>
+      <c r="AM75" s="89"/>
+      <c r="AN75" s="90"/>
       <c r="AO75" s="16"/>
       <c r="AP75" s="29"/>
       <c r="AQ75" s="26"/>
       <c r="AR75" s="24"/>
     </row>
-    <row r="76" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="12"/>
       <c r="B76" s="66" t="s">
         <v>39</v>
@@ -6187,7 +6191,7 @@
       <c r="AQ76" s="26"/>
       <c r="AR76" s="24"/>
     </row>
-    <row r="77" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="16"/>
       <c r="B77" s="69" t="s">
         <v>30</v>
@@ -6245,7 +6249,7 @@
       <c r="AQ77" s="26"/>
       <c r="AR77" s="24"/>
     </row>
-    <row r="78" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="16"/>
       <c r="B78" s="72"/>
       <c r="C78" s="73"/>
@@ -6291,7 +6295,7 @@
       <c r="AQ78" s="26"/>
       <c r="AR78" s="24"/>
     </row>
-    <row r="79" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="16"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -6337,7 +6341,7 @@
       <c r="AQ79" s="26"/>
       <c r="AR79" s="24"/>
     </row>
-    <row r="80" spans="1:44" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:44" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="12"/>
       <c r="B80" s="75" t="s">
         <v>42</v>
@@ -6353,47 +6357,47 @@
       <c r="K80" s="76"/>
       <c r="L80" s="59"/>
       <c r="M80" s="5"/>
-      <c r="N80" s="83" t="s">
+      <c r="N80" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="O80" s="84"/>
+      <c r="O80" s="87"/>
       <c r="P80" s="34"/>
       <c r="Q80" s="44"/>
-      <c r="R80" s="83" t="s">
+      <c r="R80" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="S80" s="84"/>
+      <c r="S80" s="87"/>
       <c r="T80" s="34"/>
       <c r="U80" s="36"/>
-      <c r="V80" s="83"/>
-      <c r="W80" s="84"/>
+      <c r="V80" s="86"/>
+      <c r="W80" s="87"/>
       <c r="X80" s="34"/>
       <c r="Y80" s="32"/>
-      <c r="Z80" s="83" t="s">
+      <c r="Z80" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="AA80" s="84"/>
+      <c r="AA80" s="87"/>
       <c r="AB80" s="34"/>
       <c r="AC80" s="36"/>
-      <c r="AD80" s="83" t="s">
+      <c r="AD80" s="86" t="s">
         <v>42</v>
       </c>
-      <c r="AE80" s="84"/>
+      <c r="AE80" s="87"/>
       <c r="AF80" s="34"/>
       <c r="AG80" s="32"/>
-      <c r="AH80" s="83"/>
-      <c r="AI80" s="84"/>
+      <c r="AH80" s="86"/>
+      <c r="AI80" s="87"/>
       <c r="AJ80" s="34"/>
       <c r="AK80" s="32"/>
-      <c r="AL80" s="83"/>
-      <c r="AM80" s="84"/>
+      <c r="AL80" s="86"/>
+      <c r="AM80" s="87"/>
       <c r="AN80" s="34"/>
       <c r="AO80" s="12"/>
       <c r="AP80" s="29"/>
       <c r="AQ80" s="26"/>
       <c r="AR80" s="24"/>
     </row>
-    <row r="81" spans="1:44" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:44" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="12"/>
       <c r="B81" s="63"/>
       <c r="C81" s="64"/>
@@ -6407,39 +6411,39 @@
       <c r="K81" s="64"/>
       <c r="L81" s="65"/>
       <c r="M81" s="5"/>
-      <c r="N81" s="85"/>
-      <c r="O81" s="86"/>
-      <c r="P81" s="87"/>
+      <c r="N81" s="88"/>
+      <c r="O81" s="89"/>
+      <c r="P81" s="90"/>
       <c r="Q81" s="44"/>
-      <c r="R81" s="85"/>
-      <c r="S81" s="86"/>
-      <c r="T81" s="87"/>
+      <c r="R81" s="88"/>
+      <c r="S81" s="89"/>
+      <c r="T81" s="90"/>
       <c r="U81" s="32"/>
-      <c r="V81" s="85"/>
-      <c r="W81" s="86"/>
-      <c r="X81" s="87"/>
+      <c r="V81" s="88"/>
+      <c r="W81" s="89"/>
+      <c r="X81" s="90"/>
       <c r="Y81" s="32"/>
-      <c r="Z81" s="85"/>
-      <c r="AA81" s="86"/>
-      <c r="AB81" s="87"/>
+      <c r="Z81" s="88"/>
+      <c r="AA81" s="89"/>
+      <c r="AB81" s="90"/>
       <c r="AC81" s="36"/>
-      <c r="AD81" s="85"/>
-      <c r="AE81" s="86"/>
-      <c r="AF81" s="87"/>
+      <c r="AD81" s="88"/>
+      <c r="AE81" s="89"/>
+      <c r="AF81" s="90"/>
       <c r="AG81" s="32"/>
-      <c r="AH81" s="85"/>
-      <c r="AI81" s="86"/>
-      <c r="AJ81" s="87"/>
+      <c r="AH81" s="88"/>
+      <c r="AI81" s="89"/>
+      <c r="AJ81" s="90"/>
       <c r="AK81" s="35"/>
-      <c r="AL81" s="85"/>
-      <c r="AM81" s="86"/>
-      <c r="AN81" s="87"/>
+      <c r="AL81" s="88"/>
+      <c r="AM81" s="89"/>
+      <c r="AN81" s="90"/>
       <c r="AO81" s="12"/>
       <c r="AP81" s="29"/>
       <c r="AQ81" s="26"/>
       <c r="AR81" s="24"/>
     </row>
-    <row r="82" spans="1:44" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:44" s="20" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="12"/>
       <c r="B82" s="66" t="s">
         <v>39</v>
@@ -6495,7 +6499,7 @@
       <c r="AQ82" s="26"/>
       <c r="AR82" s="24"/>
     </row>
-    <row r="83" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="12"/>
       <c r="B83" s="69" t="s">
         <v>12</v>
@@ -6551,7 +6555,7 @@
       <c r="AQ83" s="26"/>
       <c r="AR83" s="24"/>
     </row>
-    <row r="84" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A84" s="12"/>
       <c r="B84" s="72"/>
       <c r="C84" s="73"/>
@@ -6597,7 +6601,7 @@
       <c r="AQ84" s="26"/>
       <c r="AR84" s="24"/>
     </row>
-    <row r="85" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="12"/>
       <c r="B85" s="35"/>
       <c r="C85" s="35"/>
@@ -6643,7 +6647,7 @@
       <c r="AQ85" s="26"/>
       <c r="AR85" s="24"/>
     </row>
-    <row r="86" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="12"/>
       <c r="B86" s="75"/>
       <c r="C86" s="76"/>
@@ -6657,43 +6661,43 @@
       <c r="K86" s="76"/>
       <c r="L86" s="59"/>
       <c r="M86" s="6"/>
-      <c r="N86" s="83" t="s">
+      <c r="N86" s="86" t="s">
         <v>41</v>
       </c>
-      <c r="O86" s="84"/>
+      <c r="O86" s="87"/>
       <c r="P86" s="34"/>
       <c r="Q86" s="44"/>
-      <c r="R86" s="83" t="s">
+      <c r="R86" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="S86" s="84"/>
+      <c r="S86" s="87"/>
       <c r="T86" s="34"/>
       <c r="U86" s="36"/>
-      <c r="V86" s="83"/>
-      <c r="W86" s="84"/>
+      <c r="V86" s="86"/>
+      <c r="W86" s="87"/>
       <c r="X86" s="34"/>
       <c r="Y86" s="32"/>
-      <c r="Z86" s="83"/>
-      <c r="AA86" s="84"/>
+      <c r="Z86" s="86"/>
+      <c r="AA86" s="87"/>
       <c r="AB86" s="34"/>
       <c r="AC86" s="36"/>
-      <c r="AD86" s="83"/>
-      <c r="AE86" s="84"/>
+      <c r="AD86" s="86"/>
+      <c r="AE86" s="87"/>
       <c r="AF86" s="34"/>
       <c r="AG86" s="36"/>
-      <c r="AH86" s="83"/>
-      <c r="AI86" s="84"/>
+      <c r="AH86" s="86"/>
+      <c r="AI86" s="87"/>
       <c r="AJ86" s="34"/>
       <c r="AK86" s="32"/>
-      <c r="AL86" s="83"/>
-      <c r="AM86" s="84"/>
+      <c r="AL86" s="86"/>
+      <c r="AM86" s="87"/>
       <c r="AN86" s="34"/>
       <c r="AO86" s="12"/>
       <c r="AP86" s="29"/>
       <c r="AQ86" s="26"/>
       <c r="AR86" s="24"/>
     </row>
-    <row r="87" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="12"/>
       <c r="B87" s="63"/>
       <c r="C87" s="64"/>
@@ -6707,39 +6711,39 @@
       <c r="K87" s="64"/>
       <c r="L87" s="65"/>
       <c r="M87" s="6"/>
-      <c r="N87" s="85"/>
-      <c r="O87" s="86"/>
-      <c r="P87" s="87"/>
+      <c r="N87" s="88"/>
+      <c r="O87" s="89"/>
+      <c r="P87" s="90"/>
       <c r="Q87" s="44"/>
-      <c r="R87" s="85"/>
-      <c r="S87" s="86"/>
-      <c r="T87" s="87"/>
+      <c r="R87" s="88"/>
+      <c r="S87" s="89"/>
+      <c r="T87" s="90"/>
       <c r="U87" s="32"/>
-      <c r="V87" s="85"/>
-      <c r="W87" s="86"/>
-      <c r="X87" s="87"/>
+      <c r="V87" s="88"/>
+      <c r="W87" s="89"/>
+      <c r="X87" s="90"/>
       <c r="Y87" s="32"/>
-      <c r="Z87" s="85"/>
-      <c r="AA87" s="86"/>
-      <c r="AB87" s="87"/>
+      <c r="Z87" s="88"/>
+      <c r="AA87" s="89"/>
+      <c r="AB87" s="90"/>
       <c r="AC87" s="36"/>
-      <c r="AD87" s="85"/>
-      <c r="AE87" s="86"/>
-      <c r="AF87" s="87"/>
+      <c r="AD87" s="88"/>
+      <c r="AE87" s="89"/>
+      <c r="AF87" s="90"/>
       <c r="AG87" s="38"/>
-      <c r="AH87" s="85"/>
-      <c r="AI87" s="86"/>
-      <c r="AJ87" s="87"/>
+      <c r="AH87" s="88"/>
+      <c r="AI87" s="89"/>
+      <c r="AJ87" s="90"/>
       <c r="AK87" s="35"/>
-      <c r="AL87" s="85"/>
-      <c r="AM87" s="86"/>
-      <c r="AN87" s="87"/>
+      <c r="AL87" s="88"/>
+      <c r="AM87" s="89"/>
+      <c r="AN87" s="90"/>
       <c r="AO87" s="12"/>
       <c r="AP87" s="29"/>
       <c r="AQ87" s="26"/>
       <c r="AR87" s="24"/>
     </row>
-    <row r="88" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="12"/>
       <c r="B88" s="66"/>
       <c r="C88" s="67"/>
@@ -6789,7 +6793,7 @@
       <c r="AQ88" s="26"/>
       <c r="AR88" s="24"/>
     </row>
-    <row r="89" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="12"/>
       <c r="B89" s="69"/>
       <c r="C89" s="70"/>
@@ -6839,7 +6843,7 @@
       <c r="AQ89" s="26"/>
       <c r="AR89" s="24"/>
     </row>
-    <row r="90" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="12"/>
       <c r="B90" s="72"/>
       <c r="C90" s="73"/>
@@ -6885,7 +6889,7 @@
       <c r="AQ90" s="26"/>
       <c r="AR90" s="24"/>
     </row>
-    <row r="91" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="12"/>
       <c r="B91" s="35"/>
       <c r="C91" s="35"/>
@@ -6931,7 +6935,7 @@
       <c r="AQ91" s="26"/>
       <c r="AR91" s="24"/>
     </row>
-    <row r="92" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="12"/>
       <c r="B92" s="75"/>
       <c r="C92" s="76"/>
@@ -6945,39 +6949,39 @@
       <c r="K92" s="76"/>
       <c r="L92" s="59"/>
       <c r="M92" s="6"/>
-      <c r="N92" s="83"/>
-      <c r="O92" s="84"/>
+      <c r="N92" s="86"/>
+      <c r="O92" s="87"/>
       <c r="P92" s="34"/>
       <c r="Q92" s="32"/>
-      <c r="R92" s="83"/>
-      <c r="S92" s="84"/>
+      <c r="R92" s="86"/>
+      <c r="S92" s="87"/>
       <c r="T92" s="34"/>
       <c r="U92" s="36"/>
-      <c r="V92" s="83"/>
-      <c r="W92" s="84"/>
+      <c r="V92" s="86"/>
+      <c r="W92" s="87"/>
       <c r="X92" s="34"/>
       <c r="Y92" s="32"/>
-      <c r="Z92" s="83"/>
-      <c r="AA92" s="84"/>
+      <c r="Z92" s="86"/>
+      <c r="AA92" s="87"/>
       <c r="AB92" s="34"/>
       <c r="AC92" s="44"/>
-      <c r="AD92" s="83"/>
-      <c r="AE92" s="84"/>
+      <c r="AD92" s="86"/>
+      <c r="AE92" s="87"/>
       <c r="AF92" s="34"/>
       <c r="AG92" s="44"/>
-      <c r="AH92" s="83"/>
-      <c r="AI92" s="84"/>
+      <c r="AH92" s="86"/>
+      <c r="AI92" s="87"/>
       <c r="AJ92" s="34"/>
       <c r="AK92" s="32"/>
-      <c r="AL92" s="83"/>
-      <c r="AM92" s="84"/>
+      <c r="AL92" s="86"/>
+      <c r="AM92" s="87"/>
       <c r="AN92" s="34"/>
       <c r="AO92" s="12"/>
       <c r="AP92" s="29"/>
       <c r="AQ92" s="26"/>
       <c r="AR92" s="24"/>
     </row>
-    <row r="93" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="12"/>
       <c r="B93" s="63"/>
       <c r="C93" s="64"/>
@@ -6991,39 +6995,39 @@
       <c r="K93" s="64"/>
       <c r="L93" s="65"/>
       <c r="M93" s="6"/>
-      <c r="N93" s="85"/>
-      <c r="O93" s="86"/>
-      <c r="P93" s="87"/>
+      <c r="N93" s="88"/>
+      <c r="O93" s="89"/>
+      <c r="P93" s="90"/>
       <c r="Q93" s="35"/>
-      <c r="R93" s="85"/>
-      <c r="S93" s="86"/>
-      <c r="T93" s="87"/>
+      <c r="R93" s="88"/>
+      <c r="S93" s="89"/>
+      <c r="T93" s="90"/>
       <c r="U93" s="36"/>
-      <c r="V93" s="85"/>
-      <c r="W93" s="86"/>
-      <c r="X93" s="87"/>
+      <c r="V93" s="88"/>
+      <c r="W93" s="89"/>
+      <c r="X93" s="90"/>
       <c r="Y93" s="32"/>
-      <c r="Z93" s="85"/>
-      <c r="AA93" s="86"/>
-      <c r="AB93" s="87"/>
+      <c r="Z93" s="88"/>
+      <c r="AA93" s="89"/>
+      <c r="AB93" s="90"/>
       <c r="AC93" s="43"/>
-      <c r="AD93" s="85"/>
-      <c r="AE93" s="86"/>
-      <c r="AF93" s="87"/>
+      <c r="AD93" s="88"/>
+      <c r="AE93" s="89"/>
+      <c r="AF93" s="90"/>
       <c r="AG93" s="43"/>
-      <c r="AH93" s="85"/>
-      <c r="AI93" s="86"/>
-      <c r="AJ93" s="87"/>
+      <c r="AH93" s="88"/>
+      <c r="AI93" s="89"/>
+      <c r="AJ93" s="90"/>
       <c r="AK93" s="35"/>
-      <c r="AL93" s="85"/>
-      <c r="AM93" s="86"/>
-      <c r="AN93" s="87"/>
+      <c r="AL93" s="88"/>
+      <c r="AM93" s="89"/>
+      <c r="AN93" s="90"/>
       <c r="AO93" s="12"/>
       <c r="AP93" s="29"/>
       <c r="AQ93" s="26"/>
       <c r="AR93" s="24"/>
     </row>
-    <row r="94" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="12"/>
       <c r="B94" s="66"/>
       <c r="C94" s="67"/>
@@ -7069,7 +7073,7 @@
       <c r="AQ94" s="26"/>
       <c r="AR94" s="24"/>
     </row>
-    <row r="95" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="12"/>
       <c r="B95" s="69"/>
       <c r="C95" s="70"/>
@@ -7115,7 +7119,7 @@
       <c r="AQ95" s="26"/>
       <c r="AR95" s="24"/>
     </row>
-    <row r="96" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A96" s="12"/>
       <c r="B96" s="72"/>
       <c r="C96" s="73"/>
@@ -7161,7 +7165,7 @@
       <c r="AQ96" s="26"/>
       <c r="AR96" s="24"/>
     </row>
-    <row r="97" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="12"/>
       <c r="B97" s="35"/>
       <c r="C97" s="35"/>
@@ -7207,7 +7211,7 @@
       <c r="AQ97" s="26"/>
       <c r="AR97" s="24"/>
     </row>
-    <row r="98" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="12"/>
       <c r="B98" s="75"/>
       <c r="C98" s="76"/>
@@ -7221,47 +7225,47 @@
       <c r="K98" s="76"/>
       <c r="L98" s="59"/>
       <c r="M98" s="26"/>
-      <c r="N98" s="101" t="s">
+      <c r="N98" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="O98" s="102"/>
+      <c r="O98" s="105"/>
       <c r="P98" s="62"/>
       <c r="Q98" s="32"/>
-      <c r="R98" s="101" t="s">
+      <c r="R98" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="S98" s="102"/>
+      <c r="S98" s="105"/>
       <c r="T98" s="62"/>
       <c r="U98" s="36"/>
-      <c r="V98" s="101" t="s">
+      <c r="V98" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="W98" s="102"/>
+      <c r="W98" s="105"/>
       <c r="X98" s="62"/>
       <c r="Y98" s="32"/>
-      <c r="Z98" s="101" t="s">
+      <c r="Z98" s="104" t="s">
         <v>45</v>
       </c>
-      <c r="AA98" s="102"/>
+      <c r="AA98" s="105"/>
       <c r="AB98" s="62"/>
       <c r="AC98" s="36"/>
-      <c r="AD98" s="83"/>
-      <c r="AE98" s="84"/>
+      <c r="AD98" s="86"/>
+      <c r="AE98" s="87"/>
       <c r="AF98" s="34"/>
       <c r="AG98" s="32"/>
-      <c r="AH98" s="83"/>
-      <c r="AI98" s="84"/>
+      <c r="AH98" s="86"/>
+      <c r="AI98" s="87"/>
       <c r="AJ98" s="34"/>
       <c r="AK98" s="32"/>
-      <c r="AL98" s="83"/>
-      <c r="AM98" s="84"/>
+      <c r="AL98" s="86"/>
+      <c r="AM98" s="87"/>
       <c r="AN98" s="34"/>
       <c r="AO98" s="12"/>
       <c r="AP98" s="29"/>
       <c r="AQ98" s="26"/>
       <c r="AR98" s="24"/>
     </row>
-    <row r="99" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="12"/>
       <c r="B99" s="63"/>
       <c r="C99" s="64"/>
@@ -7299,23 +7303,23 @@
       <c r="AA99" s="99"/>
       <c r="AB99" s="100"/>
       <c r="AC99" s="36"/>
-      <c r="AD99" s="85"/>
-      <c r="AE99" s="86"/>
-      <c r="AF99" s="87"/>
+      <c r="AD99" s="88"/>
+      <c r="AE99" s="89"/>
+      <c r="AF99" s="90"/>
       <c r="AG99" s="32"/>
-      <c r="AH99" s="85"/>
-      <c r="AI99" s="86"/>
-      <c r="AJ99" s="87"/>
+      <c r="AH99" s="88"/>
+      <c r="AI99" s="89"/>
+      <c r="AJ99" s="90"/>
       <c r="AK99" s="35"/>
-      <c r="AL99" s="85"/>
-      <c r="AM99" s="86"/>
-      <c r="AN99" s="87"/>
+      <c r="AL99" s="88"/>
+      <c r="AM99" s="89"/>
+      <c r="AN99" s="90"/>
       <c r="AO99" s="12"/>
       <c r="AP99" s="29"/>
       <c r="AQ99" s="26"/>
       <c r="AR99" s="24"/>
     </row>
-    <row r="100" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="12"/>
       <c r="B100" s="66"/>
       <c r="C100" s="67"/>
@@ -7329,21 +7333,21 @@
       <c r="K100" s="67"/>
       <c r="L100" s="68"/>
       <c r="M100" s="26"/>
-      <c r="N100" s="103"/>
-      <c r="O100" s="104"/>
-      <c r="P100" s="105"/>
+      <c r="N100" s="101"/>
+      <c r="O100" s="102"/>
+      <c r="P100" s="103"/>
       <c r="Q100" s="31"/>
-      <c r="R100" s="103"/>
-      <c r="S100" s="104"/>
-      <c r="T100" s="105"/>
+      <c r="R100" s="101"/>
+      <c r="S100" s="102"/>
+      <c r="T100" s="103"/>
       <c r="U100" s="31"/>
-      <c r="V100" s="103"/>
-      <c r="W100" s="104"/>
-      <c r="X100" s="105"/>
+      <c r="V100" s="101"/>
+      <c r="W100" s="102"/>
+      <c r="X100" s="103"/>
       <c r="Y100" s="32"/>
-      <c r="Z100" s="103"/>
-      <c r="AA100" s="104"/>
-      <c r="AB100" s="105"/>
+      <c r="Z100" s="101"/>
+      <c r="AA100" s="102"/>
+      <c r="AB100" s="103"/>
       <c r="AC100" s="36"/>
       <c r="AD100" s="91"/>
       <c r="AE100" s="92"/>
@@ -7361,7 +7365,7 @@
       <c r="AQ100" s="26"/>
       <c r="AR100" s="24"/>
     </row>
-    <row r="101" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="12"/>
       <c r="B101" s="69"/>
       <c r="C101" s="70"/>
@@ -7415,7 +7419,7 @@
       <c r="AQ101" s="26"/>
       <c r="AR101" s="24"/>
     </row>
-    <row r="102" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A102" s="12"/>
       <c r="B102" s="72"/>
       <c r="C102" s="73"/>
@@ -7461,7 +7465,7 @@
       <c r="AQ102" s="26"/>
       <c r="AR102" s="24"/>
     </row>
-    <row r="103" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:44" s="19" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="12"/>
       <c r="B103" s="40"/>
       <c r="C103" s="33"/>
@@ -7507,7 +7511,7 @@
       <c r="AQ103" s="26"/>
       <c r="AR103" s="26"/>
     </row>
-    <row r="104" spans="1:44" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:44" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B104" s="33"/>
       <c r="C104" s="33"/>
       <c r="D104" s="33"/>
@@ -7524,34 +7528,34 @@
       <c r="AQ104" s="26"/>
       <c r="AR104" s="26"/>
     </row>
-    <row r="105" spans="1:44" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B105" s="83"/>
-      <c r="C105" s="84"/>
+    <row r="105" spans="1:44" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B105" s="86"/>
+      <c r="C105" s="87"/>
       <c r="D105" s="34"/>
       <c r="E105" s="32"/>
-      <c r="F105" s="83"/>
-      <c r="G105" s="84"/>
+      <c r="F105" s="86"/>
+      <c r="G105" s="87"/>
       <c r="H105" s="34"/>
       <c r="I105" s="32"/>
-      <c r="J105" s="83"/>
-      <c r="K105" s="84"/>
+      <c r="J105" s="86"/>
+      <c r="K105" s="87"/>
       <c r="L105" s="34"/>
       <c r="AO105" s="26"/>
     </row>
-    <row r="106" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B106" s="85"/>
-      <c r="C106" s="86"/>
-      <c r="D106" s="87"/>
+    <row r="106" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B106" s="88"/>
+      <c r="C106" s="89"/>
+      <c r="D106" s="90"/>
       <c r="E106" s="32"/>
-      <c r="F106" s="85"/>
-      <c r="G106" s="86"/>
-      <c r="H106" s="87"/>
+      <c r="F106" s="88"/>
+      <c r="G106" s="89"/>
+      <c r="H106" s="90"/>
       <c r="I106" s="32"/>
-      <c r="J106" s="85"/>
-      <c r="K106" s="86"/>
-      <c r="L106" s="87"/>
-    </row>
-    <row r="107" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J106" s="88"/>
+      <c r="K106" s="89"/>
+      <c r="L106" s="90"/>
+    </row>
+    <row r="107" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B107" s="91"/>
       <c r="C107" s="92"/>
       <c r="D107" s="93"/>
@@ -7564,7 +7568,7 @@
       <c r="K107" s="92"/>
       <c r="L107" s="93"/>
     </row>
-    <row r="108" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B108" s="69"/>
       <c r="C108" s="70"/>
       <c r="D108" s="71"/>
@@ -7577,7 +7581,7 @@
       <c r="K108" s="70"/>
       <c r="L108" s="71"/>
     </row>
-    <row r="109" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B109" s="72"/>
       <c r="C109" s="73"/>
       <c r="D109" s="74"/>
@@ -7590,7 +7594,7 @@
       <c r="K109" s="73"/>
       <c r="L109" s="74"/>
     </row>
-    <row r="110" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B110" s="35"/>
       <c r="C110" s="35"/>
       <c r="D110" s="35"/>
@@ -7603,33 +7607,33 @@
       <c r="K110" s="35"/>
       <c r="L110" s="35"/>
     </row>
-    <row r="111" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B111" s="83"/>
-      <c r="C111" s="84"/>
+    <row r="111" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B111" s="86"/>
+      <c r="C111" s="87"/>
       <c r="D111" s="34"/>
       <c r="E111" s="31"/>
-      <c r="F111" s="83"/>
-      <c r="G111" s="84"/>
+      <c r="F111" s="86"/>
+      <c r="G111" s="87"/>
       <c r="H111" s="34"/>
       <c r="I111" s="31"/>
-      <c r="J111" s="83"/>
-      <c r="K111" s="84"/>
+      <c r="J111" s="86"/>
+      <c r="K111" s="87"/>
       <c r="L111" s="34"/>
     </row>
-    <row r="112" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B112" s="85"/>
-      <c r="C112" s="86"/>
-      <c r="D112" s="87"/>
+    <row r="112" spans="1:44" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B112" s="88"/>
+      <c r="C112" s="89"/>
+      <c r="D112" s="90"/>
       <c r="E112" s="32"/>
-      <c r="F112" s="85"/>
-      <c r="G112" s="86"/>
-      <c r="H112" s="87"/>
+      <c r="F112" s="88"/>
+      <c r="G112" s="89"/>
+      <c r="H112" s="90"/>
       <c r="I112" s="32"/>
-      <c r="J112" s="85"/>
-      <c r="K112" s="86"/>
-      <c r="L112" s="87"/>
-    </row>
-    <row r="113" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J112" s="88"/>
+      <c r="K112" s="89"/>
+      <c r="L112" s="90"/>
+    </row>
+    <row r="113" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B113" s="91"/>
       <c r="C113" s="92"/>
       <c r="D113" s="93"/>
@@ -7642,7 +7646,7 @@
       <c r="K113" s="92"/>
       <c r="L113" s="93"/>
     </row>
-    <row r="114" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B114" s="69"/>
       <c r="C114" s="70"/>
       <c r="D114" s="71"/>
@@ -7655,7 +7659,7 @@
       <c r="K114" s="70"/>
       <c r="L114" s="71"/>
     </row>
-    <row r="115" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B115" s="72"/>
       <c r="C115" s="73"/>
       <c r="D115" s="74"/>
@@ -7668,7 +7672,7 @@
       <c r="K115" s="73"/>
       <c r="L115" s="74"/>
     </row>
-    <row r="116" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B116" s="35"/>
       <c r="C116" s="35"/>
       <c r="D116" s="35"/>
@@ -7681,33 +7685,33 @@
       <c r="K116" s="35"/>
       <c r="L116" s="35"/>
     </row>
-    <row r="117" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="83"/>
-      <c r="C117" s="84"/>
+    <row r="117" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B117" s="86"/>
+      <c r="C117" s="87"/>
       <c r="D117" s="34"/>
       <c r="E117" s="32"/>
-      <c r="F117" s="83"/>
-      <c r="G117" s="84"/>
+      <c r="F117" s="86"/>
+      <c r="G117" s="87"/>
       <c r="H117" s="34"/>
       <c r="I117" s="32"/>
-      <c r="J117" s="83"/>
-      <c r="K117" s="84"/>
+      <c r="J117" s="86"/>
+      <c r="K117" s="87"/>
       <c r="L117" s="34"/>
     </row>
-    <row r="118" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="85"/>
-      <c r="C118" s="86"/>
-      <c r="D118" s="87"/>
+    <row r="118" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B118" s="88"/>
+      <c r="C118" s="89"/>
+      <c r="D118" s="90"/>
       <c r="E118" s="32"/>
-      <c r="F118" s="85"/>
-      <c r="G118" s="86"/>
-      <c r="H118" s="87"/>
+      <c r="F118" s="88"/>
+      <c r="G118" s="89"/>
+      <c r="H118" s="90"/>
       <c r="I118" s="32"/>
-      <c r="J118" s="85"/>
-      <c r="K118" s="86"/>
-      <c r="L118" s="87"/>
-    </row>
-    <row r="119" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J118" s="88"/>
+      <c r="K118" s="89"/>
+      <c r="L118" s="90"/>
+    </row>
+    <row r="119" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B119" s="91"/>
       <c r="C119" s="92"/>
       <c r="D119" s="93"/>
@@ -7720,7 +7724,7 @@
       <c r="K119" s="92"/>
       <c r="L119" s="93"/>
     </row>
-    <row r="120" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B120" s="69"/>
       <c r="C120" s="70"/>
       <c r="D120" s="71"/>
@@ -7733,7 +7737,7 @@
       <c r="K120" s="70"/>
       <c r="L120" s="71"/>
     </row>
-    <row r="121" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B121" s="72"/>
       <c r="C121" s="73"/>
       <c r="D121" s="74"/>
@@ -7746,7 +7750,7 @@
       <c r="K121" s="73"/>
       <c r="L121" s="74"/>
     </row>
-    <row r="122" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B122" s="35"/>
       <c r="C122" s="35"/>
       <c r="D122" s="35"/>
@@ -7759,33 +7763,33 @@
       <c r="K122" s="35"/>
       <c r="L122" s="35"/>
     </row>
-    <row r="123" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B123" s="83"/>
-      <c r="C123" s="84"/>
+    <row r="123" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B123" s="86"/>
+      <c r="C123" s="87"/>
       <c r="D123" s="34"/>
       <c r="E123" s="32"/>
-      <c r="F123" s="83"/>
-      <c r="G123" s="84"/>
+      <c r="F123" s="86"/>
+      <c r="G123" s="87"/>
       <c r="H123" s="34"/>
       <c r="I123" s="32"/>
-      <c r="J123" s="83"/>
-      <c r="K123" s="84"/>
+      <c r="J123" s="86"/>
+      <c r="K123" s="87"/>
       <c r="L123" s="34"/>
     </row>
-    <row r="124" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B124" s="85"/>
-      <c r="C124" s="86"/>
-      <c r="D124" s="87"/>
+    <row r="124" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B124" s="88"/>
+      <c r="C124" s="89"/>
+      <c r="D124" s="90"/>
       <c r="E124" s="32"/>
-      <c r="F124" s="85"/>
-      <c r="G124" s="86"/>
-      <c r="H124" s="87"/>
+      <c r="F124" s="88"/>
+      <c r="G124" s="89"/>
+      <c r="H124" s="90"/>
       <c r="I124" s="32"/>
-      <c r="J124" s="85"/>
-      <c r="K124" s="86"/>
-      <c r="L124" s="87"/>
-    </row>
-    <row r="125" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J124" s="88"/>
+      <c r="K124" s="89"/>
+      <c r="L124" s="90"/>
+    </row>
+    <row r="125" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B125" s="91"/>
       <c r="C125" s="92"/>
       <c r="D125" s="93"/>
@@ -7798,7 +7802,7 @@
       <c r="K125" s="92"/>
       <c r="L125" s="93"/>
     </row>
-    <row r="126" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B126" s="69"/>
       <c r="C126" s="70"/>
       <c r="D126" s="71"/>
@@ -7811,7 +7815,7 @@
       <c r="K126" s="70"/>
       <c r="L126" s="71"/>
     </row>
-    <row r="127" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B127" s="72"/>
       <c r="C127" s="73"/>
       <c r="D127" s="74"/>
@@ -7824,7 +7828,7 @@
       <c r="K127" s="73"/>
       <c r="L127" s="74"/>
     </row>
-    <row r="128" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B128" s="35"/>
       <c r="C128" s="35"/>
       <c r="D128" s="35"/>
@@ -7837,33 +7841,33 @@
       <c r="K128" s="35"/>
       <c r="L128" s="35"/>
     </row>
-    <row r="129" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B129" s="83"/>
-      <c r="C129" s="84"/>
+    <row r="129" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B129" s="86"/>
+      <c r="C129" s="87"/>
       <c r="D129" s="34"/>
       <c r="E129" s="31"/>
-      <c r="F129" s="83"/>
-      <c r="G129" s="84"/>
+      <c r="F129" s="86"/>
+      <c r="G129" s="87"/>
       <c r="H129" s="34"/>
       <c r="I129" s="32"/>
-      <c r="J129" s="83"/>
-      <c r="K129" s="84"/>
+      <c r="J129" s="86"/>
+      <c r="K129" s="87"/>
       <c r="L129" s="34"/>
     </row>
-    <row r="130" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B130" s="85"/>
-      <c r="C130" s="86"/>
-      <c r="D130" s="87"/>
+    <row r="130" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B130" s="88"/>
+      <c r="C130" s="89"/>
+      <c r="D130" s="90"/>
       <c r="E130" s="32"/>
-      <c r="F130" s="85"/>
-      <c r="G130" s="86"/>
-      <c r="H130" s="87"/>
+      <c r="F130" s="88"/>
+      <c r="G130" s="89"/>
+      <c r="H130" s="90"/>
       <c r="I130" s="32"/>
-      <c r="J130" s="85"/>
-      <c r="K130" s="86"/>
-      <c r="L130" s="87"/>
-    </row>
-    <row r="131" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J130" s="88"/>
+      <c r="K130" s="89"/>
+      <c r="L130" s="90"/>
+    </row>
+    <row r="131" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B131" s="91"/>
       <c r="C131" s="92"/>
       <c r="D131" s="93"/>
@@ -7876,7 +7880,7 @@
       <c r="K131" s="92"/>
       <c r="L131" s="93"/>
     </row>
-    <row r="132" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B132" s="69"/>
       <c r="C132" s="70"/>
       <c r="D132" s="71"/>
@@ -7889,7 +7893,7 @@
       <c r="K132" s="70"/>
       <c r="L132" s="71"/>
     </row>
-    <row r="133" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:12" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B133" s="72"/>
       <c r="C133" s="73"/>
       <c r="D133" s="74"/>
@@ -7927,6 +7931,8 @@
     <mergeCell ref="B64:D64"/>
     <mergeCell ref="F64:H64"/>
     <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="F52:H52"/>
     <mergeCell ref="AD50:AF50"/>
     <mergeCell ref="AD52:AE52"/>
     <mergeCell ref="V47:X47"/>
@@ -7951,8 +7957,6 @@
     <mergeCell ref="F48:H48"/>
     <mergeCell ref="F49:H49"/>
     <mergeCell ref="J69:L69"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="F52:H52"/>
     <mergeCell ref="AD90:AF90"/>
     <mergeCell ref="AD93:AF93"/>
     <mergeCell ref="AD94:AF94"/>
@@ -7972,6 +7976,10 @@
     <mergeCell ref="AD87:AF87"/>
     <mergeCell ref="AD88:AF88"/>
     <mergeCell ref="AD89:AF89"/>
+    <mergeCell ref="Z69:AB69"/>
+    <mergeCell ref="Z70:AB70"/>
+    <mergeCell ref="AD84:AF84"/>
+    <mergeCell ref="AD83:AF83"/>
     <mergeCell ref="B76:D76"/>
     <mergeCell ref="B70:D70"/>
     <mergeCell ref="J70:L70"/>
@@ -8006,8 +8014,20 @@
     <mergeCell ref="J54:L54"/>
     <mergeCell ref="N54:P54"/>
     <mergeCell ref="F54:H54"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:P52"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="J59:L59"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="N63:P63"/>
+    <mergeCell ref="N61:P61"/>
+    <mergeCell ref="Z64:AB64"/>
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="J53:L53"/>
     <mergeCell ref="V54:X54"/>
@@ -8020,20 +8040,16 @@
     <mergeCell ref="R52:T52"/>
     <mergeCell ref="R58:S58"/>
     <mergeCell ref="R59:T59"/>
-    <mergeCell ref="N49:P49"/>
-    <mergeCell ref="J48:L48"/>
-    <mergeCell ref="R53:T53"/>
-    <mergeCell ref="R49:T49"/>
-    <mergeCell ref="N47:P47"/>
-    <mergeCell ref="N53:P53"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:P38"/>
-    <mergeCell ref="R37:S37"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="J40:L40"/>
-    <mergeCell ref="J49:L49"/>
-    <mergeCell ref="N44:P44"/>
-    <mergeCell ref="N45:P45"/>
+    <mergeCell ref="J63:L63"/>
+    <mergeCell ref="J56:L56"/>
+    <mergeCell ref="F60:H60"/>
+    <mergeCell ref="J60:L60"/>
+    <mergeCell ref="J55:L55"/>
+    <mergeCell ref="J61:L61"/>
+    <mergeCell ref="J62:L62"/>
+    <mergeCell ref="F56:H56"/>
+    <mergeCell ref="F55:H55"/>
+    <mergeCell ref="F58:G58"/>
     <mergeCell ref="J52:L52"/>
     <mergeCell ref="J47:L47"/>
     <mergeCell ref="J46:L46"/>
@@ -8042,27 +8058,8 @@
     <mergeCell ref="R43:S43"/>
     <mergeCell ref="R44:T44"/>
     <mergeCell ref="R45:T45"/>
-    <mergeCell ref="J63:L63"/>
-    <mergeCell ref="J56:L56"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="F60:H60"/>
-    <mergeCell ref="J60:L60"/>
-    <mergeCell ref="J55:L55"/>
-    <mergeCell ref="J61:L61"/>
-    <mergeCell ref="J62:L62"/>
-    <mergeCell ref="F56:H56"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="F55:H55"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="J59:L59"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:P52"/>
     <mergeCell ref="J106:L106"/>
     <mergeCell ref="Z100:AB100"/>
     <mergeCell ref="N92:O92"/>
@@ -8135,6 +8132,8 @@
     <mergeCell ref="V88:X88"/>
     <mergeCell ref="V89:X89"/>
     <mergeCell ref="R90:T90"/>
+    <mergeCell ref="Z88:AB88"/>
+    <mergeCell ref="R88:T88"/>
     <mergeCell ref="B126:D126"/>
     <mergeCell ref="F126:H126"/>
     <mergeCell ref="J126:L126"/>
@@ -8232,7 +8231,6 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="AH10:AJ10"/>
     <mergeCell ref="R27:S27"/>
-    <mergeCell ref="J16:L16"/>
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="Z12:AA12"/>
@@ -8251,14 +8249,6 @@
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="F13:H13"/>
     <mergeCell ref="J13:L13"/>
-    <mergeCell ref="Z20:AA20"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="R16:T16"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="N18:AB19"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="V20:W20"/>
     <mergeCell ref="F62:H62"/>
     <mergeCell ref="F61:H61"/>
     <mergeCell ref="Z23:AA23"/>
@@ -8275,11 +8265,33 @@
     <mergeCell ref="N33:P33"/>
     <mergeCell ref="N41:P41"/>
     <mergeCell ref="V33:X33"/>
-    <mergeCell ref="N63:P63"/>
-    <mergeCell ref="N61:P61"/>
-    <mergeCell ref="AH31:AI31"/>
-    <mergeCell ref="AD32:AF32"/>
-    <mergeCell ref="AD46:AF46"/>
+    <mergeCell ref="N49:P49"/>
+    <mergeCell ref="J48:L48"/>
+    <mergeCell ref="R53:T53"/>
+    <mergeCell ref="R49:T49"/>
+    <mergeCell ref="N47:P47"/>
+    <mergeCell ref="N53:P53"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:P38"/>
+    <mergeCell ref="AD41:AF41"/>
+    <mergeCell ref="AD33:AF33"/>
+    <mergeCell ref="R35:T35"/>
+    <mergeCell ref="R34:T34"/>
+    <mergeCell ref="R41:T41"/>
+    <mergeCell ref="R40:T40"/>
+    <mergeCell ref="V27:W27"/>
+    <mergeCell ref="Z20:AA20"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="R16:T16"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="N18:AB19"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="V20:W20"/>
+    <mergeCell ref="J16:L16"/>
+    <mergeCell ref="R37:S37"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="J40:L40"/>
     <mergeCell ref="AD20:AE20"/>
     <mergeCell ref="AH20:AI20"/>
     <mergeCell ref="N20:O20"/>
@@ -8293,11 +8305,6 @@
     <mergeCell ref="Z21:AA21"/>
     <mergeCell ref="V32:X32"/>
     <mergeCell ref="Z32:AB32"/>
-    <mergeCell ref="AD40:AF40"/>
-    <mergeCell ref="AD41:AF41"/>
-    <mergeCell ref="AD33:AF33"/>
-    <mergeCell ref="AH48:AJ48"/>
-    <mergeCell ref="AH46:AJ46"/>
     <mergeCell ref="AD27:AE27"/>
     <mergeCell ref="AH54:AJ54"/>
     <mergeCell ref="AD54:AF54"/>
@@ -8317,6 +8324,11 @@
     <mergeCell ref="AH74:AI74"/>
     <mergeCell ref="AH71:AJ71"/>
     <mergeCell ref="AD57:AF57"/>
+    <mergeCell ref="AH40:AJ40"/>
+    <mergeCell ref="AH31:AI31"/>
+    <mergeCell ref="AD32:AF32"/>
+    <mergeCell ref="AD46:AF46"/>
+    <mergeCell ref="AD40:AF40"/>
     <mergeCell ref="B106:D106"/>
     <mergeCell ref="F106:H106"/>
     <mergeCell ref="F105:G105"/>
@@ -8551,10 +8563,6 @@
     <mergeCell ref="V83:X83"/>
     <mergeCell ref="Z81:AB81"/>
     <mergeCell ref="V77:X77"/>
-    <mergeCell ref="Z88:AB88"/>
-    <mergeCell ref="N81:P81"/>
-    <mergeCell ref="N83:P83"/>
-    <mergeCell ref="N76:P76"/>
     <mergeCell ref="N55:P55"/>
     <mergeCell ref="R56:T56"/>
     <mergeCell ref="V78:X78"/>
@@ -8571,16 +8579,9 @@
     <mergeCell ref="V74:W74"/>
     <mergeCell ref="V60:X60"/>
     <mergeCell ref="R55:T55"/>
-    <mergeCell ref="R88:T88"/>
     <mergeCell ref="R75:T75"/>
     <mergeCell ref="V68:W68"/>
     <mergeCell ref="R63:T63"/>
-    <mergeCell ref="Z64:AB64"/>
-    <mergeCell ref="Z69:AB69"/>
-    <mergeCell ref="Z70:AB70"/>
-    <mergeCell ref="AD84:AF84"/>
-    <mergeCell ref="AD83:AF83"/>
-    <mergeCell ref="AH40:AJ40"/>
     <mergeCell ref="N86:O86"/>
     <mergeCell ref="R86:S86"/>
     <mergeCell ref="Z87:AB87"/>
@@ -8594,6 +8595,9 @@
     <mergeCell ref="V72:X72"/>
     <mergeCell ref="Z72:AB72"/>
     <mergeCell ref="Z71:AB71"/>
+    <mergeCell ref="N81:P81"/>
+    <mergeCell ref="N83:P83"/>
+    <mergeCell ref="N76:P76"/>
     <mergeCell ref="AH80:AI80"/>
     <mergeCell ref="AH82:AJ82"/>
     <mergeCell ref="AH81:AJ81"/>
@@ -8606,12 +8610,8 @@
     <mergeCell ref="Z44:AB44"/>
     <mergeCell ref="Z45:AB45"/>
     <mergeCell ref="AD36:AF36"/>
-    <mergeCell ref="R35:T35"/>
-    <mergeCell ref="R34:T34"/>
-    <mergeCell ref="R41:T41"/>
     <mergeCell ref="Z41:AB41"/>
     <mergeCell ref="Z40:AB40"/>
-    <mergeCell ref="R40:T40"/>
     <mergeCell ref="AH38:AI38"/>
     <mergeCell ref="AH42:AJ42"/>
     <mergeCell ref="AH43:AJ43"/>
@@ -8620,6 +8620,8 @@
     <mergeCell ref="AH45:AI45"/>
     <mergeCell ref="AD43:AF43"/>
     <mergeCell ref="AD45:AE45"/>
+    <mergeCell ref="AH48:AJ48"/>
+    <mergeCell ref="AH46:AJ46"/>
     <mergeCell ref="AL34:AN34"/>
     <mergeCell ref="AL35:AN35"/>
     <mergeCell ref="AL39:AN39"/>
@@ -8688,7 +8690,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="F26:G26"/>
-    <mergeCell ref="V27:W27"/>
     <mergeCell ref="Z27:AA27"/>
     <mergeCell ref="V35:X35"/>
     <mergeCell ref="V39:X39"/>
@@ -8704,6 +8705,8 @@
     <mergeCell ref="V38:X38"/>
     <mergeCell ref="R38:T38"/>
     <mergeCell ref="N35:P35"/>
+    <mergeCell ref="N44:P44"/>
+    <mergeCell ref="N45:P45"/>
     <mergeCell ref="N21:O21"/>
     <mergeCell ref="R21:S21"/>
     <mergeCell ref="F40:H40"/>
@@ -8770,6 +8773,7 @@
     <mergeCell ref="J51:K51"/>
     <mergeCell ref="F46:H46"/>
     <mergeCell ref="B46:D46"/>
+    <mergeCell ref="J49:L49"/>
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="B88:D88"/>
     <mergeCell ref="B89:D89"/>
@@ -8792,7 +8796,7 @@
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="P22:P27 X22:X27 AB22:AB27 AJ22:AJ27 AF22:AF27 AN22:AN27 T22:T27 L22:L27 H22:H27 D22:D27">
       <formula1>$AP$68:$AP$71</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="R46:T49 AH14:AJ16 AL22:AM27 V95:X96 AD77:AF78 R22:S27 V77:X78 J132:L133 AL71:AN72 AH48:AJ50 N77:P78 Z95:AB96 R71:T72 N95:P96 AD71:AF72 Z46:AB49 V22:W27 AD48:AF50 AL101:AN102 J14:L16 V8:X10 V46:X49 AD95:AF96 J114:L115 AD8:AF10 AL89:AN90 AH95:AJ96 R8:T10 N46:P49 B108:D109 N54:P56 Z14:AB16 R54:T56 R14:T16 R101:T102 AL14:AN16 AH83:AJ84 R34:T35 V54:X56 AD41:AF43 R89:T90 J120:L121 F114:H115 F126:H127 F132:H133 B120:D121 J108:L109 F120:H121 B132:D133 B126:D127 AD14:AF16 B114:D115 J126:L127 V34:X35 V101:X102 V61:X64 AL83:AN84 AH89:AJ90 AD22:AE27 V14:X16 AD89:AF90 F108:H109 Z89:AB90 N22:O27 J95:L96 AL48:AN50 R61:T64 AH55:AJ57 J8:L10 N34:P35 Z54:AB56 R77:T78 AH22:AI27 N61:P64 AL41:AN43 B14:D16 J77:L78 AD101:AF102 N14:P16 R95:T96 AH8:AJ10 R40:T41 AH34:AJ36 AH62:AJ64 Z101:AB102 AD55:AF57 Z77:AB78 Z83:AB84 N71:P72 V83:X84 Z34:AB35 Z22:AA27 AD83:AF84 Z61:AB64 AH71:AJ72 AH101:AJ102 Z40:AB41 AL77:AN78 AL62:AN64 Z8:AB10 V40:X41 AL8:AN10 N40:P41 N8:P10 AD62:AF64 Z71:AB72 AL95:AN96 AD34:AF36 F22:G27 R83:T84 V89:X90 AL34:AN36 N83:P84 F14:H16 B22:C27 J22:K27 F89:H90 F95:H96 V71:X72 AH41:AJ43 AL55:AN57 B89:D90 J101:L102 B95:D96 B8:D10 J89:L90 F8:H10 F101:H102 AH77:AJ78 B101:D102 N89:P90 J71:L72 J46:L49 B71:D72 B40:D41 F40:H41 F34:H35 J83:L84 F46:H49 J54:L56 J34:L35 J61:L64 B54:D56 B77:D78 J40:L41 F54:H56 F77:H78 B34:D35 F83:H84 B46:D49 F71:H72 B61:D64 F61:H64 B83:D84 N101:P102">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Yazım Hatası" error="İstanbul Ses Servisinde olmayan bir isim girdiniz." promptTitle="uuuuuuuuuu" prompt="yyyyyyyyyyyy" sqref="R46:T49 AH14:AJ16 AL22:AM27 V95:X96 AD77:AF78 R22:S27 V77:X78 J132:L133 AL71:AN72 N101:P102 N77:P78 Z95:AB96 R71:T72 N95:P96 AD71:AF72 Z46:AB49 V22:W27 AD48:AF50 AL101:AN102 J14:L16 V8:X10 V46:X49 AD95:AF96 J114:L115 AD8:AF10 AL89:AN90 AH95:AJ96 R8:T10 N46:P49 B108:D109 N54:P56 Z14:AB16 R54:T56 R14:T16 R101:T102 AL14:AN16 AH83:AJ84 R34:T35 V54:X56 AD41:AF43 R89:T90 J120:L121 F114:H115 F126:H127 F132:H133 B120:D121 J108:L109 F120:H121 B132:D133 B126:D127 AD14:AF16 B114:D115 J126:L127 V34:X35 V101:X102 V61:X64 AL83:AN84 AH89:AJ90 AD22:AE27 V14:X16 AD89:AF90 F108:H109 Z89:AB90 N22:O27 J95:L96 AL48:AN50 R61:T64 AH55:AJ57 J8:L10 N34:P35 Z54:AB56 R77:T78 AH22:AI27 N61:P64 AL41:AN43 B14:D16 J77:L78 AD101:AF102 N14:P16 R95:T96 AH8:AJ10 R40:T41 AD34:AF36 AH62:AJ64 Z101:AB102 AD55:AF57 Z77:AB78 Z83:AB84 N71:P72 V83:X84 Z34:AB35 Z22:AA27 AD83:AF84 Z61:AB64 AH71:AJ72 AH101:AJ102 Z40:AB41 AL77:AN78 AL62:AN64 Z8:AB10 V40:X41 AL8:AN10 N40:P41 N8:P10 AD62:AF64 Z71:AB72 AL95:AN96 AH48:AJ50 F22:G27 R83:T84 V89:X90 AL34:AN36 N83:P84 F14:H16 B22:C27 J22:K27 F89:H90 F95:H96 V71:X72 AH41:AJ43 AL55:AN57 B89:D90 J101:L102 B95:D96 B8:D10 J89:L90 F8:H10 F101:H102 AH77:AJ78 B101:D102 N89:P90 J71:L72 J46:L49 B71:D72 B40:D41 F40:H41 F34:H35 J83:L84 F46:H49 J54:L56 J34:L35 J61:L64 B54:D56 B77:D78 J40:L41 F54:H56 F77:H78 B34:D35 F83:H84 B46:D49 F71:H72 B61:D64 F61:H64 B83:D84 AH34:AJ36">
       <formula1>$AP$6:$AP$30</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>